<commit_message>
DONE: Corrected red FPGA comparison csv and added RGB FPGA comparison csv.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_Red.xlsx
+++ b/FPGA_Performance_Comparison_Red.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB160863-78C4-914C-8332-EBD4A8170443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B0AE40-B6FB-294D-A67B-D83DD6E1F871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17860" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="-10500" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
   <si>
     <t>FPGA Implementation</t>
   </si>
@@ -213,13 +213,46 @@
   </si>
   <si>
     <t>% Change From Standard</t>
+  </si>
+  <si>
+    <t>First Pixel Out</t>
+  </si>
+  <si>
+    <t>Last Pixel Out</t>
+  </si>
+  <si>
+    <t>First Pixel In</t>
+  </si>
+  <si>
+    <t>Last Pixel In</t>
+  </si>
+  <si>
+    <t>Input To Output Programmed Latency (Clock Cycles)</t>
+  </si>
+  <si>
+    <t>Computation Programmed Latency (Clock Cycles)</t>
+  </si>
+  <si>
+    <t>Input To Output Programmed Latency (ms)</t>
+  </si>
+  <si>
+    <t>Computation Programmed Latency (us)</t>
+  </si>
+  <si>
+    <t>Programmed Energy Per Frame (uJ)</t>
+  </si>
+  <si>
+    <t>17x128x128</t>
+  </si>
+  <si>
+    <t>Light Field Dimensions (Sub-Apertures, Length, Width)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -230,6 +263,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -262,11 +301,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -279,9 +315,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -292,12 +325,26 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -634,68 +681,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45085A3-2BCA-FA4F-9A9B-A0D6975F9A68}">
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="50.83203125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="50.83203125" style="3" customWidth="1"/>
     <col min="2" max="4" width="25.83203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" style="11"/>
-    <col min="6" max="7" width="25.83203125" style="12" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="11"/>
+    <col min="6" max="7" width="25.83203125" style="1" customWidth="1"/>
     <col min="9" max="10" width="25.83203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="2" t="s">
+      <c r="G1" s="9"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="8"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="10"/>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="6" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="6" t="s">
+      <c r="H2" s="6"/>
+      <c r="I2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="8"/>
+      <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="1">
@@ -707,7 +751,7 @@
       <c r="D3" s="1">
         <v>200</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="1">
         <f>C3-B3</f>
         <v>0</v>
@@ -716,19 +760,19 @@
         <f>D3-B3</f>
         <v>120</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="7">
+      <c r="H3" s="6"/>
+      <c r="I3" s="5">
         <f>F3/B3</f>
         <v>0</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="5">
         <f>G3/B3</f>
         <v>1.5</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="1">
@@ -740,7 +784,7 @@
       <c r="D4" s="1">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="1">
         <f t="shared" ref="F4:F5" si="0">C4-B4</f>
         <v>4.3940000000000001</v>
@@ -749,19 +793,19 @@
         <f t="shared" ref="G4:G5" si="1">D4-B4</f>
         <v>-0.20799999999999999</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="7">
+      <c r="H4" s="6"/>
+      <c r="I4" s="5">
         <f t="shared" ref="I4:I5" si="2">F4/B4</f>
         <v>17.93469387755102</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="5">
         <f t="shared" ref="J4:J5" si="3">G4/B4</f>
         <v>-0.84897959183673466</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="1">
@@ -773,7 +817,7 @@
       <c r="D5" s="1">
         <v>201.53</v>
       </c>
-      <c r="E5" s="8"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="1">
         <f t="shared" si="0"/>
         <v>45.620000000000005</v>
@@ -782,32 +826,32 @@
         <f t="shared" si="1"/>
         <v>119.92</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="7">
+      <c r="H5" s="6"/>
+      <c r="I5" s="5">
         <f t="shared" si="2"/>
         <v>0.55900012253400322</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="5">
         <f t="shared" si="3"/>
         <v>1.4694277662051221</v>
       </c>
-      <c r="K5" s="8"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="8"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1">
@@ -819,7 +863,7 @@
       <c r="D7" s="1">
         <v>11914</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="1">
         <f>C7-B7</f>
         <v>-57</v>
@@ -828,19 +872,19 @@
         <f>D7-B7</f>
         <v>67</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="7">
+      <c r="H7" s="6"/>
+      <c r="I7" s="5">
         <f>F7/B7</f>
         <v>-4.8113446442137253E-3</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="5">
         <f>G7/B7</f>
         <v>5.6554401958301683E-3</v>
       </c>
-      <c r="K7" s="8"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1">
@@ -852,7 +896,7 @@
       <c r="D8" s="1">
         <v>30828</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="1">
         <f>C8-B8</f>
         <v>866</v>
@@ -861,19 +905,19 @@
         <f>D8-B8</f>
         <v>3743</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="7">
+      <c r="H8" s="6"/>
+      <c r="I8" s="5">
         <f>F8/B8</f>
         <v>3.1973417020491043E-2</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="5">
         <f>G8/B8</f>
         <v>0.13819457264168358</v>
       </c>
-      <c r="K8" s="8"/>
+      <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="1">
@@ -885,7 +929,7 @@
       <c r="D9" s="1">
         <v>3199112</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="1">
         <f>C9-B9</f>
         <v>-36</v>
@@ -894,65 +938,61 @@
         <f>D9-B9</f>
         <v>-36</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="7">
+      <c r="H9" s="6"/>
+      <c r="I9" s="5">
         <f>F9/B9</f>
         <v>-1.1252996110214344E-5</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="5">
         <f>G9/B9</f>
         <v>-1.1252996110214344E-5</v>
       </c>
-      <c r="K9" s="8"/>
+      <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="9">
         <v>12</v>
       </c>
-      <c r="C10" s="1">
-        <v>12</v>
-      </c>
-      <c r="D10" s="1">
-        <v>12</v>
-      </c>
-      <c r="E10" s="8"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="1">
         <f>C10-B10</f>
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="G10" s="1">
         <f>D10-B10</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="7">
+        <v>-12</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="5">
         <f>F10/B10</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="7">
+        <v>-1</v>
+      </c>
+      <c r="J10" s="5">
         <f>G10/B10</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="8"/>
+        <v>-1</v>
+      </c>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="8"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="1">
@@ -964,28 +1004,28 @@
       <c r="D12" s="1">
         <v>1386.71</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="1">
-        <f>C12-B12</f>
+        <f t="shared" ref="F12:F31" si="4">C12-B12</f>
         <v>-10.529999999999973</v>
       </c>
       <c r="G12" s="1">
-        <f>D12-B12</f>
+        <f t="shared" ref="G12:G31" si="5">D12-B12</f>
         <v>589.97</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="7">
-        <f>F12/B12</f>
+      <c r="H12" s="6"/>
+      <c r="I12" s="5">
+        <f t="shared" ref="I12:I31" si="6">F12/B12</f>
         <v>-1.3216356653362418E-2</v>
       </c>
-      <c r="J12" s="7">
-        <f>G12/B12</f>
+      <c r="J12" s="5">
+        <f t="shared" ref="J12:J31" si="7">G12/B12</f>
         <v>0.7404799558199664</v>
       </c>
-      <c r="K12" s="8"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="1">
@@ -997,28 +1037,28 @@
       <c r="D13" s="1">
         <v>948.92</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="1">
-        <f>C13-B13</f>
+        <f t="shared" si="4"/>
         <v>-10.5</v>
       </c>
       <c r="G13" s="1">
-        <f>D13-B13</f>
+        <f t="shared" si="5"/>
         <v>582.59999999999991</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="7">
-        <f>F13/B13</f>
+      <c r="H13" s="6"/>
+      <c r="I13" s="5">
+        <f t="shared" si="6"/>
         <v>-2.8663463638348985E-2</v>
       </c>
-      <c r="J13" s="7">
-        <f>G13/B13</f>
+      <c r="J13" s="5">
+        <f t="shared" si="7"/>
         <v>1.5904127538763919</v>
       </c>
-      <c r="K13" s="8"/>
+      <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B14" s="1">
@@ -1030,28 +1070,28 @@
       <c r="D14" s="1">
         <v>421.09</v>
       </c>
-      <c r="E14" s="8"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="1">
-        <f>C14-B14</f>
+        <f t="shared" si="4"/>
         <v>-6.9999999999993179E-2</v>
       </c>
       <c r="G14" s="1">
-        <f>D14-B14</f>
+        <f t="shared" si="5"/>
         <v>3.7199999999999704</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="7">
-        <f>F14/B14</f>
+      <c r="H14" s="6"/>
+      <c r="I14" s="5">
+        <f t="shared" si="6"/>
         <v>-1.6771689388310894E-4</v>
       </c>
-      <c r="J14" s="7">
-        <f>G14/B14</f>
+      <c r="J14" s="5">
+        <f t="shared" si="7"/>
         <v>8.9129549320745866E-3</v>
       </c>
-      <c r="K14" s="8"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="1">
@@ -1063,28 +1103,28 @@
       <c r="D15" s="1">
         <v>16.7</v>
       </c>
-      <c r="E15" s="8"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="1">
-        <f>C15-B15</f>
+        <f t="shared" si="4"/>
         <v>2.9999999999999361E-2</v>
       </c>
       <c r="G15" s="1">
-        <f>D15-B15</f>
+        <f t="shared" si="5"/>
         <v>3.6499999999999986</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="7">
-        <f>F15/B15</f>
+      <c r="H15" s="6"/>
+      <c r="I15" s="5">
+        <f t="shared" si="6"/>
         <v>2.2988505747125946E-3</v>
       </c>
-      <c r="J15" s="7">
-        <f>G15/B15</f>
+      <c r="J15" s="5">
+        <f t="shared" si="7"/>
         <v>0.27969348659003818</v>
       </c>
-      <c r="K15" s="8"/>
+      <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="1">
@@ -1096,28 +1136,28 @@
       <c r="D16" s="1">
         <v>957.61</v>
       </c>
-      <c r="E16" s="8"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="1">
-        <f>C16-B16</f>
+        <f t="shared" si="4"/>
         <v>-10.470000000000027</v>
       </c>
       <c r="G16" s="1">
-        <f>D16-B16</f>
+        <f t="shared" si="5"/>
         <v>586.24</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="7">
-        <f>F16/B16</f>
+      <c r="H16" s="6"/>
+      <c r="I16" s="5">
+        <f t="shared" si="6"/>
         <v>-2.8192907343081098E-2</v>
       </c>
-      <c r="J16" s="7">
-        <f>G16/B16</f>
+      <c r="J16" s="5">
+        <f t="shared" si="7"/>
         <v>1.5785873926272989</v>
       </c>
-      <c r="K16" s="8"/>
+      <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B17" s="1">
@@ -1129,28 +1169,28 @@
       <c r="D17" s="1">
         <v>644.32000000000005</v>
       </c>
-      <c r="E17" s="8"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="1">
-        <f>C17-B17</f>
+        <f t="shared" si="4"/>
         <v>-0.11999999999997613</v>
       </c>
       <c r="G17" s="1">
-        <f>D17-B17</f>
+        <f t="shared" si="5"/>
         <v>394.59000000000003</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="7">
-        <f>F17/B17</f>
+      <c r="H17" s="6"/>
+      <c r="I17" s="5">
+        <f t="shared" si="6"/>
         <v>-4.8051896047721993E-4</v>
       </c>
-      <c r="J17" s="7">
-        <f>G17/B17</f>
+      <c r="J17" s="5">
+        <f t="shared" si="7"/>
         <v>1.580066471789533</v>
       </c>
-      <c r="K17" s="8"/>
+      <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="1">
@@ -1162,28 +1202,28 @@
       <c r="D18" s="1">
         <v>42.25</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="1">
-        <f>C18-B18</f>
+        <f t="shared" si="4"/>
         <v>0.32000000000000028</v>
       </c>
       <c r="G18" s="1">
-        <f>D18-B18</f>
+        <f t="shared" si="5"/>
         <v>24.72</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="7">
-        <f>F18/B18</f>
+      <c r="H18" s="6"/>
+      <c r="I18" s="5">
+        <f t="shared" si="6"/>
         <v>1.8254420992584158E-2</v>
       </c>
-      <c r="J18" s="7">
-        <f>G18/B18</f>
+      <c r="J18" s="5">
+        <f t="shared" si="7"/>
         <v>1.4101540216771247</v>
       </c>
-      <c r="K18" s="8"/>
+      <c r="K18" s="6"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="1">
@@ -1195,28 +1235,28 @@
       <c r="D19" s="1">
         <v>34.729999999999997</v>
       </c>
-      <c r="E19" s="8"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="1">
-        <f>C19-B19</f>
+        <f t="shared" si="4"/>
         <v>0.12999999999999901</v>
       </c>
       <c r="G19" s="1">
-        <f>D19-B19</f>
+        <f t="shared" si="5"/>
         <v>21.58</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="7">
-        <f>F19/B19</f>
+      <c r="H19" s="6"/>
+      <c r="I19" s="5">
+        <f t="shared" si="6"/>
         <v>9.8859315589352858E-3</v>
       </c>
-      <c r="J19" s="7">
-        <f>G19/B19</f>
+      <c r="J19" s="5">
+        <f t="shared" si="7"/>
         <v>1.6410646387832697</v>
       </c>
-      <c r="K19" s="8"/>
+      <c r="K19" s="6"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="1">
@@ -1228,28 +1268,28 @@
       <c r="D20" s="1">
         <v>180.76</v>
       </c>
-      <c r="E20" s="8"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="1">
-        <f>C20-B20</f>
+        <f t="shared" si="4"/>
         <v>-2.6899999999999977</v>
       </c>
       <c r="G20" s="1">
-        <f>D20-B20</f>
+        <f t="shared" si="5"/>
         <v>-23.25</v>
       </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="7">
-        <f>F20/B20</f>
+      <c r="H20" s="6"/>
+      <c r="I20" s="5">
+        <f t="shared" si="6"/>
         <v>-1.3185628155482564E-2</v>
       </c>
-      <c r="J20" s="7">
-        <f>G20/B20</f>
+      <c r="J20" s="5">
+        <f t="shared" si="7"/>
         <v>-0.11396500171560218</v>
       </c>
-      <c r="K20" s="8"/>
+      <c r="K20" s="6"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B21" s="1">
@@ -1261,28 +1301,28 @@
       <c r="D21" s="1">
         <v>147.25</v>
       </c>
-      <c r="E21" s="8"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="1">
-        <f>C21-B21</f>
+        <f t="shared" si="4"/>
         <v>-0.43999999999999773</v>
       </c>
       <c r="G21" s="1">
-        <f>D21-B21</f>
+        <f t="shared" si="5"/>
         <v>-39.620000000000005</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="7">
-        <f>F21/B21</f>
+      <c r="H21" s="6"/>
+      <c r="I21" s="5">
+        <f t="shared" si="6"/>
         <v>-2.3545780489109954E-3</v>
       </c>
-      <c r="J21" s="7">
-        <f>G21/B21</f>
+      <c r="J21" s="5">
+        <f t="shared" si="7"/>
         <v>-0.21201905067694121</v>
       </c>
-      <c r="K21" s="8"/>
+      <c r="K21" s="6"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="1">
@@ -1294,28 +1334,28 @@
       <c r="D22" s="1">
         <v>333.91</v>
       </c>
-      <c r="E22" s="8"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="1">
-        <f>C22-B22</f>
+        <f t="shared" si="4"/>
         <v>-0.12000000000000011</v>
       </c>
       <c r="G22" s="1">
-        <f>D22-B22</f>
+        <f t="shared" si="5"/>
         <v>330.71000000000004</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="7">
-        <f>F22/B22</f>
+      <c r="H22" s="6"/>
+      <c r="I22" s="5">
+        <f t="shared" si="6"/>
         <v>-3.7500000000000033E-2</v>
       </c>
-      <c r="J22" s="7">
-        <f>G22/B22</f>
+      <c r="J22" s="5">
+        <f t="shared" si="7"/>
         <v>103.34687500000001</v>
       </c>
-      <c r="K22" s="8"/>
+      <c r="K22" s="6"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="1">
@@ -1327,28 +1367,28 @@
       <c r="D23" s="1">
         <v>325.57</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="6"/>
       <c r="F23" s="1">
-        <f>C23-B23</f>
+        <f t="shared" si="4"/>
         <v>-4.0000000000000036E-2</v>
       </c>
       <c r="G23" s="1">
-        <f>D23-B23</f>
+        <f t="shared" si="5"/>
         <v>324.3</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="7">
-        <f>F23/B23</f>
+      <c r="H23" s="6"/>
+      <c r="I23" s="5">
+        <f t="shared" si="6"/>
         <v>-3.1496062992126012E-2</v>
       </c>
-      <c r="J23" s="7">
-        <f>G23/B23</f>
+      <c r="J23" s="5">
+        <f t="shared" si="7"/>
         <v>255.35433070866142</v>
       </c>
-      <c r="K23" s="8"/>
+      <c r="K23" s="6"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B24" s="1">
@@ -1360,28 +1400,28 @@
       <c r="D24" s="1">
         <v>2.9</v>
       </c>
-      <c r="E24" s="8"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="1">
-        <f>C24-B24</f>
+        <f t="shared" si="4"/>
         <v>1.0000000000000009E-2</v>
       </c>
       <c r="G24" s="1">
-        <f>D24-B24</f>
+        <f t="shared" si="5"/>
         <v>1.96</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="7">
-        <f>F24/B24</f>
+      <c r="H24" s="6"/>
+      <c r="I24" s="5">
+        <f t="shared" si="6"/>
         <v>1.0638297872340436E-2</v>
       </c>
-      <c r="J24" s="7">
-        <f>G24/B24</f>
+      <c r="J24" s="5">
+        <f t="shared" si="7"/>
         <v>2.0851063829787235</v>
       </c>
-      <c r="K24" s="8"/>
+      <c r="K24" s="6"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="1">
@@ -1393,28 +1433,28 @@
       <c r="D25" s="1">
         <v>1.22</v>
       </c>
-      <c r="E25" s="8"/>
+      <c r="E25" s="6"/>
       <c r="F25" s="1">
-        <f>C25-B25</f>
+        <f t="shared" si="4"/>
         <v>1.0000000000000009E-2</v>
       </c>
       <c r="G25" s="1">
-        <f>D25-B25</f>
+        <f t="shared" si="5"/>
         <v>0.83</v>
       </c>
-      <c r="H25" s="8"/>
-      <c r="I25" s="7">
-        <f>F25/B25</f>
+      <c r="H25" s="6"/>
+      <c r="I25" s="5">
+        <f t="shared" si="6"/>
         <v>2.5641025641025664E-2</v>
       </c>
-      <c r="J25" s="7">
-        <f>G25/B25</f>
+      <c r="J25" s="5">
+        <f t="shared" si="7"/>
         <v>2.1282051282051282</v>
       </c>
-      <c r="K25" s="8"/>
+      <c r="K25" s="6"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B26" s="1">
@@ -1426,28 +1466,28 @@
       <c r="D26" s="1">
         <v>190.96</v>
       </c>
-      <c r="E26" s="8"/>
+      <c r="E26" s="6"/>
       <c r="F26" s="1">
-        <f>C26-B26</f>
+        <f t="shared" si="4"/>
         <v>-0.44000000000000483</v>
       </c>
       <c r="G26" s="1">
-        <f>D26-B26</f>
+        <f t="shared" si="5"/>
         <v>126.65</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="7">
-        <f>F26/B26</f>
+      <c r="H26" s="6"/>
+      <c r="I26" s="5">
+        <f t="shared" si="6"/>
         <v>-6.8418597418753663E-3</v>
       </c>
-      <c r="J26" s="7">
-        <f>G26/B26</f>
+      <c r="J26" s="5">
+        <f t="shared" si="7"/>
         <v>1.9693671279738765</v>
       </c>
-      <c r="K26" s="8"/>
+      <c r="K26" s="6"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="1">
@@ -1459,28 +1499,28 @@
       <c r="D27" s="1">
         <v>87.22</v>
       </c>
-      <c r="E27" s="8"/>
+      <c r="E27" s="6"/>
       <c r="F27" s="1">
-        <f>C27-B27</f>
+        <f t="shared" si="4"/>
         <v>1.0299999999999976</v>
       </c>
       <c r="G27" s="1">
-        <f>D27-B27</f>
+        <f t="shared" si="5"/>
         <v>57.709999999999994</v>
       </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="7">
-        <f>F27/B27</f>
+      <c r="H27" s="6"/>
+      <c r="I27" s="5">
+        <f t="shared" si="6"/>
         <v>3.4903422568620723E-2</v>
       </c>
-      <c r="J27" s="7">
-        <f>G27/B27</f>
+      <c r="J27" s="5">
+        <f t="shared" si="7"/>
         <v>1.9556082683835985</v>
       </c>
-      <c r="K27" s="8"/>
+      <c r="K27" s="6"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B28" s="1">
@@ -1492,28 +1532,28 @@
       <c r="D28" s="1">
         <v>17.350000000000001</v>
       </c>
-      <c r="E28" s="8"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="1">
-        <f>C28-B28</f>
+        <f t="shared" si="4"/>
         <v>-0.76000000000000068</v>
       </c>
       <c r="G28" s="1">
-        <f>D28-B28</f>
+        <f t="shared" si="5"/>
         <v>11.490000000000002</v>
       </c>
-      <c r="H28" s="8"/>
-      <c r="I28" s="7">
-        <f>F28/B28</f>
+      <c r="H28" s="6"/>
+      <c r="I28" s="5">
+        <f t="shared" si="6"/>
         <v>-0.12969283276450522</v>
       </c>
-      <c r="J28" s="7">
-        <f>G28/B28</f>
+      <c r="J28" s="5">
+        <f t="shared" si="7"/>
         <v>1.960750853242321</v>
       </c>
-      <c r="K28" s="8"/>
+      <c r="K28" s="6"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="1">
@@ -1525,28 +1565,28 @@
       <c r="D29" s="1">
         <v>12.79</v>
       </c>
-      <c r="E29" s="8"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="1">
-        <f>C29-B29</f>
+        <f t="shared" si="4"/>
         <v>-0.55000000000000027</v>
       </c>
       <c r="G29" s="1">
-        <f>D29-B29</f>
+        <f t="shared" si="5"/>
         <v>8.4199999999999982</v>
       </c>
-      <c r="H29" s="8"/>
-      <c r="I29" s="7">
-        <f>F29/B29</f>
+      <c r="H29" s="6"/>
+      <c r="I29" s="5">
+        <f t="shared" si="6"/>
         <v>-0.12585812356979412</v>
       </c>
-      <c r="J29" s="7">
-        <f>G29/B29</f>
+      <c r="J29" s="5">
+        <f t="shared" si="7"/>
         <v>1.9267734553775739</v>
       </c>
-      <c r="K29" s="8"/>
-    </row>
-    <row r="30" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+      <c r="K29" s="6"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="1">
@@ -1558,28 +1598,28 @@
       <c r="D30" s="1">
         <v>66.86</v>
       </c>
-      <c r="E30" s="8"/>
+      <c r="E30" s="6"/>
       <c r="F30" s="1">
-        <f>C30-B30</f>
+        <f t="shared" si="4"/>
         <v>-2.0900000000000034</v>
       </c>
       <c r="G30" s="1">
-        <f>D30-B30</f>
+        <f t="shared" si="5"/>
         <v>40.69</v>
       </c>
-      <c r="H30" s="8"/>
-      <c r="I30" s="7">
-        <f>F30/B30</f>
+      <c r="H30" s="6"/>
+      <c r="I30" s="5">
+        <f t="shared" si="6"/>
         <v>-7.9862437905999367E-2</v>
       </c>
-      <c r="J30" s="7">
-        <f>G30/B30</f>
+      <c r="J30" s="5">
+        <f t="shared" si="7"/>
         <v>1.5548337791364155</v>
       </c>
-      <c r="K30" s="8"/>
+      <c r="K30" s="6"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="1">
@@ -1591,860 +1631,1034 @@
       <c r="D31" s="1">
         <v>28.72</v>
       </c>
-      <c r="E31" s="8"/>
+      <c r="E31" s="6"/>
       <c r="F31" s="1">
-        <f>C31-B31</f>
+        <f t="shared" si="4"/>
         <v>-0.25</v>
       </c>
       <c r="G31" s="1">
-        <f>D31-B31</f>
+        <f t="shared" si="5"/>
         <v>17.149999999999999</v>
       </c>
-      <c r="H31" s="8"/>
-      <c r="I31" s="7">
-        <f>F31/B31</f>
+      <c r="H31" s="6"/>
+      <c r="I31" s="5">
+        <f t="shared" si="6"/>
         <v>-2.1607605877268798E-2</v>
       </c>
-      <c r="J31" s="7">
-        <f>G31/B31</f>
+      <c r="J31" s="5">
+        <f t="shared" si="7"/>
         <v>1.4822817631806395</v>
       </c>
-      <c r="K31" s="8"/>
+      <c r="K31" s="6"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="8"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="6"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B33" s="1">
         <v>0.47430600000000001</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="9">
         <v>2.0395829999999999</v>
       </c>
-      <c r="D33" s="1">
-        <v>2.0395829999999999</v>
-      </c>
-      <c r="E33" s="8"/>
-      <c r="F33" s="1">
+      <c r="D33" s="9"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="9">
         <f>C33-B33</f>
         <v>1.565277</v>
       </c>
-      <c r="G33" s="1">
-        <f>D33-B33</f>
-        <v>1.565277</v>
-      </c>
-      <c r="H33" s="8"/>
-      <c r="I33" s="7">
+      <c r="G33" s="9"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="13">
         <f>F33/B33</f>
         <v>3.3001416806871515</v>
       </c>
-      <c r="J33" s="7">
-        <f>G33/B33</f>
-        <v>3.3001416806871515</v>
-      </c>
-      <c r="K33" s="8"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="6"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B34" s="1">
         <v>0.346667</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="9">
         <v>0.93874999999999997</v>
       </c>
-      <c r="D34" s="1">
-        <v>0.93874999999999997</v>
-      </c>
-      <c r="E34" s="8"/>
-      <c r="F34" s="1">
-        <f t="shared" ref="F34:F44" si="4">C34-B34</f>
+      <c r="D34" s="9"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="9">
+        <f t="shared" ref="F34:F44" si="8">C34-B34</f>
         <v>0.59208299999999991</v>
       </c>
-      <c r="G34" s="1">
-        <f t="shared" ref="G34:G44" si="5">D34-B34</f>
-        <v>0.59208299999999991</v>
-      </c>
-      <c r="H34" s="8"/>
-      <c r="I34" s="7">
-        <f t="shared" ref="I34:I44" si="6">F34/B34</f>
+      <c r="G34" s="9"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="13">
+        <f t="shared" ref="I34:I44" si="9">F34/B34</f>
         <v>1.7079300885287607</v>
       </c>
-      <c r="J34" s="7">
-        <f t="shared" ref="J34:J44" si="7">G34/B34</f>
-        <v>1.7079300885287607</v>
-      </c>
-      <c r="K34" s="8"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="6"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="1">
         <v>0</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" s="9">
         <v>1</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="9"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="9">
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
-      <c r="E35" s="8"/>
-      <c r="F35" s="1">
-        <f t="shared" si="4"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="J35" s="13"/>
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1">
+        <v>0</v>
+      </c>
+      <c r="C36" s="9">
         <v>1</v>
       </c>
-      <c r="G35" s="1">
-        <f t="shared" si="5"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="9">
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
-      <c r="H35" s="8"/>
-      <c r="I35" s="7" t="s">
+      <c r="G36" s="9"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="J35" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K35" s="8"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="1">
-        <v>0</v>
-      </c>
-      <c r="C36" s="1">
-        <v>1</v>
-      </c>
-      <c r="D36" s="1">
-        <v>1</v>
-      </c>
-      <c r="E36" s="8"/>
-      <c r="F36" s="1">
-        <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="G36" s="1">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="H36" s="8"/>
-      <c r="I36" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="J36" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K36" s="8"/>
+      <c r="J36" s="13"/>
+      <c r="K36" s="6"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="1">
         <v>-3</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" s="9">
         <v>-1</v>
       </c>
-      <c r="D37" s="1">
-        <v>-1</v>
-      </c>
-      <c r="E37" s="8"/>
-      <c r="F37" s="1">
-        <f t="shared" si="4"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="9">
+        <f t="shared" si="8"/>
         <v>2</v>
       </c>
-      <c r="G37" s="1">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="H37" s="8"/>
-      <c r="I37" s="7">
-        <f t="shared" si="6"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="13">
+        <f t="shared" si="9"/>
         <v>-0.66666666666666663</v>
       </c>
-      <c r="J37" s="7">
-        <f t="shared" si="7"/>
-        <v>-0.66666666666666663</v>
-      </c>
-      <c r="K37" s="8"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="6"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B38" s="1">
         <v>1</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C38" s="9">
         <v>7</v>
       </c>
-      <c r="D38" s="1">
-        <v>7</v>
-      </c>
-      <c r="E38" s="8"/>
-      <c r="F38" s="1">
-        <f t="shared" si="4"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="9">
+        <f t="shared" si="8"/>
         <v>6</v>
       </c>
-      <c r="G38" s="1">
-        <f t="shared" si="5"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="13">
+        <f t="shared" si="9"/>
         <v>6</v>
       </c>
-      <c r="H38" s="8"/>
-      <c r="I38" s="7">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
-      <c r="J38" s="7">
-        <f t="shared" si="7"/>
-        <v>6</v>
-      </c>
-      <c r="K38" s="8"/>
+      <c r="J38" s="13"/>
+      <c r="K38" s="6"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="1">
         <v>7.6160420000000002</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="9">
         <v>7.1617360000000003</v>
       </c>
-      <c r="D39" s="1">
-        <v>7.1617360000000003</v>
-      </c>
-      <c r="E39" s="8"/>
-      <c r="F39" s="1">
-        <f t="shared" si="4"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="9">
+        <f t="shared" si="8"/>
         <v>-0.45430599999999988</v>
       </c>
-      <c r="G39" s="1">
-        <f t="shared" si="5"/>
-        <v>-0.45430599999999988</v>
-      </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="7">
-        <f t="shared" si="6"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="13">
+        <f t="shared" si="9"/>
         <v>-5.9651194150452412E-2</v>
       </c>
-      <c r="J39" s="7">
-        <f t="shared" si="7"/>
-        <v>-5.9651194150452412E-2</v>
-      </c>
-      <c r="K39" s="8"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="6"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
       <c r="B40" s="1">
         <v>8</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" s="9">
         <v>7</v>
       </c>
-      <c r="D40" s="1">
-        <v>7</v>
-      </c>
-      <c r="E40" s="8"/>
-      <c r="F40" s="1">
-        <f t="shared" si="4"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="9">
+        <f t="shared" si="8"/>
         <v>-1</v>
       </c>
-      <c r="G40" s="1">
-        <f t="shared" si="5"/>
-        <v>-1</v>
-      </c>
-      <c r="H40" s="8"/>
-      <c r="I40" s="7">
-        <f t="shared" si="6"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="13">
+        <f t="shared" si="9"/>
         <v>-0.125</v>
       </c>
-      <c r="J40" s="7">
-        <f t="shared" si="7"/>
-        <v>-0.125</v>
-      </c>
-      <c r="K40" s="8"/>
+      <c r="J40" s="13"/>
+      <c r="K40" s="6"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B41" s="1">
         <v>8</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" s="9">
         <v>8</v>
       </c>
-      <c r="D41" s="1">
-        <v>8</v>
-      </c>
-      <c r="E41" s="8"/>
-      <c r="F41" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="G41" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="H41" s="8"/>
-      <c r="I41" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J41" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="K41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="9">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="9"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="13">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="J41" s="13"/>
+      <c r="K41" s="6"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B42" s="1">
         <v>5</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42" s="9">
         <v>4</v>
       </c>
-      <c r="D42" s="1">
-        <v>4</v>
-      </c>
-      <c r="E42" s="8"/>
-      <c r="F42" s="1">
-        <f t="shared" si="4"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="9">
+        <f t="shared" si="8"/>
         <v>-1</v>
       </c>
-      <c r="G42" s="1">
-        <f t="shared" si="5"/>
-        <v>-1</v>
-      </c>
-      <c r="H42" s="8"/>
-      <c r="I42" s="7">
-        <f t="shared" si="6"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="13">
+        <f t="shared" si="9"/>
         <v>-0.2</v>
       </c>
-      <c r="J42" s="7">
-        <f t="shared" si="7"/>
-        <v>-0.2</v>
-      </c>
-      <c r="K42" s="8"/>
+      <c r="J42" s="13"/>
+      <c r="K42" s="6"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B43" s="1">
         <v>10234</v>
       </c>
-      <c r="C43" s="1">
+      <c r="C43" s="9">
         <v>6033</v>
       </c>
-      <c r="D43" s="1">
-        <v>6033</v>
-      </c>
-      <c r="E43" s="8"/>
-      <c r="F43" s="1">
-        <f t="shared" si="4"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="9">
+        <f t="shared" si="8"/>
         <v>-4201</v>
       </c>
-      <c r="G43" s="1">
-        <f t="shared" si="5"/>
-        <v>-4201</v>
-      </c>
-      <c r="H43" s="8"/>
-      <c r="I43" s="7">
-        <f t="shared" si="6"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="13">
+        <f t="shared" si="9"/>
         <v>-0.41049443033027166</v>
       </c>
-      <c r="J43" s="7">
-        <f t="shared" si="7"/>
-        <v>-0.41049443033027166</v>
-      </c>
-      <c r="K43" s="8"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="6"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="7">
+      <c r="B44" s="5">
         <v>0.71069444000000004</v>
       </c>
-      <c r="C44" s="13">
+      <c r="C44" s="12">
         <v>0.41895832999999999</v>
       </c>
-      <c r="D44" s="7">
-        <v>0.41895832999999999</v>
-      </c>
-      <c r="E44" s="8"/>
-      <c r="F44" s="1">
-        <f t="shared" si="4"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="9">
+        <f t="shared" si="8"/>
         <v>-0.29173611000000005</v>
       </c>
-      <c r="G44" s="1">
-        <f t="shared" si="5"/>
-        <v>-0.29173611000000005</v>
-      </c>
-      <c r="H44" s="8"/>
-      <c r="I44" s="7">
-        <f t="shared" si="6"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="13">
+        <f t="shared" si="9"/>
         <v>-0.41049443133394997</v>
       </c>
-      <c r="J44" s="7">
-        <f t="shared" si="7"/>
-        <v>-0.41049443133394997</v>
-      </c>
-      <c r="K44" s="8"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="6"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A45" s="9"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="10"/>
-      <c r="J45" s="10"/>
-      <c r="K45" s="8"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="6"/>
+      <c r="I45" s="8"/>
+      <c r="J45" s="8"/>
+      <c r="K45" s="6"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="1">
         <v>4.131875</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" s="9">
         <v>3.605556</v>
       </c>
-      <c r="D46" s="1">
-        <v>3.605556</v>
-      </c>
-      <c r="E46" s="8"/>
-      <c r="F46" s="1">
+      <c r="D46" s="9"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="9">
         <f>C46-B46</f>
         <v>-0.52631899999999998</v>
       </c>
-      <c r="G46" s="1">
-        <f>D46-B46</f>
-        <v>-0.52631899999999998</v>
-      </c>
-      <c r="H46" s="8"/>
-      <c r="I46" s="7">
-        <f t="shared" ref="I46" si="8">F46/B46</f>
+      <c r="G46" s="9"/>
+      <c r="H46" s="6"/>
+      <c r="I46" s="13">
+        <f t="shared" ref="I46" si="10">F46/B46</f>
         <v>-0.12738018454091665</v>
       </c>
-      <c r="J46" s="7">
-        <f t="shared" ref="J46" si="9">G46/B46</f>
-        <v>-0.12738018454091665</v>
-      </c>
-      <c r="K46" s="8"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="6"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="1">
         <v>1.9239580000000001</v>
       </c>
-      <c r="C47" s="1">
+      <c r="C47" s="9">
         <v>1.838889</v>
       </c>
-      <c r="D47" s="1">
-        <v>1.838889</v>
-      </c>
-      <c r="E47" s="8"/>
-      <c r="F47" s="1">
-        <f t="shared" ref="F47:F57" si="10">C47-B47</f>
+      <c r="D47" s="9"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="9">
+        <f t="shared" ref="F47:F57" si="11">C47-B47</f>
         <v>-8.5069000000000061E-2</v>
       </c>
-      <c r="G47" s="1">
-        <f t="shared" ref="G47:G57" si="11">D47-B47</f>
-        <v>-8.5069000000000061E-2</v>
-      </c>
-      <c r="H47" s="8"/>
-      <c r="I47" s="7">
+      <c r="G47" s="9"/>
+      <c r="H47" s="6"/>
+      <c r="I47" s="13">
         <f t="shared" ref="I47:I57" si="12">F47/B47</f>
         <v>-4.4215622170546372E-2</v>
       </c>
-      <c r="J47" s="7">
-        <f t="shared" ref="J47:J57" si="13">G47/B47</f>
-        <v>-4.4215622170546372E-2</v>
-      </c>
-      <c r="K47" s="8"/>
+      <c r="J47" s="13"/>
+      <c r="K47" s="6"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B48" s="1">
         <v>2</v>
       </c>
-      <c r="C48" s="1">
+      <c r="C48" s="9">
         <v>2</v>
       </c>
-      <c r="D48" s="1">
-        <v>2</v>
-      </c>
-      <c r="E48" s="8"/>
-      <c r="F48" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="G48" s="1">
+      <c r="D48" s="9"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="H48" s="8"/>
-      <c r="I48" s="7">
+      <c r="G48" s="9"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="13">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J48" s="7">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K48" s="8"/>
+      <c r="J48" s="13"/>
+      <c r="K48" s="6"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="1">
         <v>-2</v>
       </c>
-      <c r="C49" s="1">
+      <c r="C49" s="9">
         <v>-2</v>
       </c>
-      <c r="D49" s="1">
-        <v>-2</v>
-      </c>
-      <c r="E49" s="8"/>
-      <c r="F49" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="1">
+      <c r="D49" s="9"/>
+      <c r="E49" s="6"/>
+      <c r="F49" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="H49" s="8"/>
-      <c r="I49" s="7">
+      <c r="G49" s="9"/>
+      <c r="H49" s="6"/>
+      <c r="I49" s="13">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J49" s="7">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K49" s="8"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="6"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="1">
         <v>-3</v>
       </c>
-      <c r="C50" s="1">
+      <c r="C50" s="9">
         <v>-3</v>
       </c>
-      <c r="D50" s="1">
-        <v>-3</v>
-      </c>
-      <c r="E50" s="8"/>
-      <c r="F50" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="G50" s="1">
+      <c r="D50" s="9"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="H50" s="8"/>
-      <c r="I50" s="7">
+      <c r="G50" s="9"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="13">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J50" s="7">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K50" s="8"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="6"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="1">
         <v>19</v>
       </c>
-      <c r="C51" s="1">
+      <c r="C51" s="9">
         <v>3</v>
       </c>
-      <c r="D51" s="1">
-        <v>3</v>
-      </c>
-      <c r="E51" s="8"/>
-      <c r="F51" s="1">
-        <f t="shared" si="10"/>
-        <v>-16</v>
-      </c>
-      <c r="G51" s="1">
+      <c r="D51" s="9"/>
+      <c r="E51" s="6"/>
+      <c r="F51" s="9">
         <f t="shared" si="11"/>
         <v>-16</v>
       </c>
-      <c r="H51" s="8"/>
-      <c r="I51" s="7">
+      <c r="G51" s="9"/>
+      <c r="H51" s="6"/>
+      <c r="I51" s="13">
         <f t="shared" si="12"/>
         <v>-0.84210526315789469</v>
       </c>
-      <c r="J51" s="7">
-        <f t="shared" si="13"/>
-        <v>-0.84210526315789469</v>
-      </c>
-      <c r="K51" s="8"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="6"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="1">
         <v>6.8117359999999998</v>
       </c>
-      <c r="C52" s="1">
+      <c r="C52" s="9">
         <v>6.8386810000000002</v>
       </c>
-      <c r="D52" s="1">
-        <v>6.8386810000000002</v>
-      </c>
-      <c r="E52" s="8"/>
-      <c r="F52" s="1">
-        <f t="shared" si="10"/>
-        <v>2.6945000000000441E-2</v>
-      </c>
-      <c r="G52" s="1">
+      <c r="D52" s="9"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="9">
         <f t="shared" si="11"/>
         <v>2.6945000000000441E-2</v>
       </c>
-      <c r="H52" s="8"/>
-      <c r="I52" s="7">
+      <c r="G52" s="9"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="13">
         <f t="shared" si="12"/>
         <v>3.9556729738205419E-3</v>
       </c>
-      <c r="J52" s="7">
-        <f t="shared" si="13"/>
-        <v>3.9556729738205419E-3</v>
-      </c>
-      <c r="K52" s="8"/>
+      <c r="J52" s="13"/>
+      <c r="K52" s="6"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="1">
         <v>7</v>
       </c>
-      <c r="C53" s="1">
+      <c r="C53" s="9">
         <v>7</v>
       </c>
-      <c r="D53" s="1">
-        <v>7</v>
-      </c>
-      <c r="E53" s="8"/>
-      <c r="F53" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="G53" s="1">
+      <c r="D53" s="9"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="H53" s="8"/>
-      <c r="I53" s="7">
+      <c r="G53" s="9"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="13">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J53" s="7">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K53" s="8"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="6"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B54" s="1">
         <v>8</v>
       </c>
-      <c r="C54" s="1">
+      <c r="C54" s="9">
         <v>8</v>
       </c>
-      <c r="D54" s="1">
-        <v>8</v>
-      </c>
-      <c r="E54" s="8"/>
-      <c r="F54" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="G54" s="1">
+      <c r="D54" s="9"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="H54" s="8"/>
-      <c r="I54" s="7">
+      <c r="G54" s="9"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="13">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J54" s="7">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="K54" s="8"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="6"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B55" s="1">
         <v>4</v>
       </c>
-      <c r="C55" s="1">
+      <c r="C55" s="9">
         <v>5</v>
       </c>
-      <c r="D55" s="1">
-        <v>5</v>
-      </c>
-      <c r="E55" s="8"/>
-      <c r="F55" s="1">
-        <f t="shared" si="10"/>
-        <v>1</v>
-      </c>
-      <c r="G55" s="1">
+      <c r="D55" s="9"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="9">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
-      <c r="H55" s="8"/>
-      <c r="I55" s="7">
+      <c r="G55" s="9"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="13">
         <f t="shared" si="12"/>
         <v>0.25</v>
       </c>
-      <c r="J55" s="7">
-        <f t="shared" si="13"/>
-        <v>0.25</v>
-      </c>
-      <c r="K55" s="8"/>
+      <c r="J55" s="13"/>
+      <c r="K55" s="6"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="1">
         <v>195</v>
       </c>
-      <c r="C56" s="1">
+      <c r="C56" s="9">
         <v>274</v>
       </c>
-      <c r="D56" s="1">
-        <v>274</v>
-      </c>
-      <c r="E56" s="8"/>
-      <c r="F56" s="1">
-        <f t="shared" si="10"/>
-        <v>79</v>
-      </c>
-      <c r="G56" s="1">
+      <c r="D56" s="9"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="9">
         <f t="shared" si="11"/>
         <v>79</v>
       </c>
-      <c r="H56" s="8"/>
-      <c r="I56" s="7">
+      <c r="G56" s="9"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="13">
         <f t="shared" si="12"/>
         <v>0.40512820512820513</v>
       </c>
-      <c r="J56" s="7">
-        <f t="shared" si="13"/>
-        <v>0.40512820512820513</v>
-      </c>
-      <c r="K56" s="8"/>
+      <c r="J56" s="13"/>
+      <c r="K56" s="6"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="7">
+      <c r="B57" s="5">
         <v>1.354167E-2</v>
       </c>
-      <c r="C57" s="7">
+      <c r="C57" s="13">
         <v>1.9027780000000001E-2</v>
       </c>
-      <c r="D57" s="7">
-        <v>1.9027780000000001E-2</v>
-      </c>
-      <c r="E57" s="8"/>
-      <c r="F57" s="1">
-        <f t="shared" si="10"/>
-        <v>5.4861100000000006E-3</v>
-      </c>
-      <c r="G57" s="1">
+      <c r="D57" s="13"/>
+      <c r="E57" s="6"/>
+      <c r="F57" s="9">
         <f t="shared" si="11"/>
         <v>5.4861100000000006E-3</v>
       </c>
-      <c r="H57" s="8"/>
-      <c r="I57" s="7">
+      <c r="G57" s="9"/>
+      <c r="H57" s="6"/>
+      <c r="I57" s="13">
         <f t="shared" si="12"/>
         <v>0.405128023353102</v>
       </c>
-      <c r="J57" s="7">
-        <f t="shared" si="13"/>
-        <v>0.405128023353102</v>
-      </c>
-      <c r="K57" s="8"/>
+      <c r="J57" s="13"/>
+      <c r="K57" s="6"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A58" s="9"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="8"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="8"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
-      <c r="K58" s="8"/>
+      <c r="A58" s="7"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="8"/>
+      <c r="J58" s="8"/>
+      <c r="K58" s="6"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C59" s="14"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14"/>
+      <c r="H59" s="6"/>
+      <c r="I59" s="15">
+        <v>0</v>
+      </c>
+      <c r="J59" s="15"/>
+      <c r="K59" s="6"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" s="9">
+        <v>1</v>
+      </c>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="9">
+        <v>0</v>
+      </c>
+      <c r="G60" s="9"/>
+      <c r="H60" s="6"/>
+      <c r="I60" s="13">
+        <f t="shared" ref="I60" si="13">F60/B60</f>
+        <v>0</v>
+      </c>
+      <c r="J60" s="13"/>
+      <c r="K60" s="6"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61" s="9">
+        <v>278529</v>
+      </c>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="9">
+        <v>0</v>
+      </c>
+      <c r="G61" s="9"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="13">
+        <f t="shared" ref="I61:I63" si="14">F61/B61</f>
+        <v>0</v>
+      </c>
+      <c r="J61" s="13"/>
+      <c r="K61" s="6"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="9">
+        <v>279694</v>
+      </c>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="6"/>
+      <c r="F62" s="9">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="13">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="J62" s="13"/>
+      <c r="K62" s="6"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63" s="9">
+        <v>295045</v>
+      </c>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="9">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="13">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="J63" s="13"/>
+      <c r="K63" s="6"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B64" s="9">
+        <f>B63-B60</f>
+        <v>295044</v>
+      </c>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="9">
+        <v>0</v>
+      </c>
+      <c r="G64" s="9"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="13">
+        <f t="shared" ref="I64:I68" si="15">F64/B64</f>
+        <v>0</v>
+      </c>
+      <c r="J64" s="13"/>
+      <c r="K64" s="6"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B65" s="9">
+        <f>B64/(B3*10^3)</f>
+        <v>3.6880500000000001</v>
+      </c>
+      <c r="C65" s="9"/>
+      <c r="D65" s="1">
+        <f>B64/(D3*10^3)</f>
+        <v>1.47522</v>
+      </c>
+      <c r="E65" s="6"/>
+      <c r="F65" s="1">
+        <v>0</v>
+      </c>
+      <c r="G65" s="1">
+        <f t="shared" ref="G64:G67" si="16">D65-B65</f>
+        <v>-2.2128300000000003</v>
+      </c>
+      <c r="H65" s="6"/>
+      <c r="I65" s="5">
+        <v>0</v>
+      </c>
+      <c r="J65" s="5">
+        <f t="shared" ref="J64:J68" si="17">G65/B65</f>
+        <v>-0.60000000000000009</v>
+      </c>
+      <c r="K65" s="6"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" s="9">
+        <f>B63-B61</f>
+        <v>16516</v>
+      </c>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="9">
+        <v>0</v>
+      </c>
+      <c r="G66" s="9"/>
+      <c r="H66" s="6"/>
+      <c r="I66" s="13">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="13"/>
+      <c r="K66" s="6"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B67" s="9">
+        <f>B66/B3</f>
+        <v>206.45</v>
+      </c>
+      <c r="C67" s="9"/>
+      <c r="D67" s="1">
+        <f>B66/D3</f>
+        <v>82.58</v>
+      </c>
+      <c r="E67" s="6"/>
+      <c r="F67" s="1">
+        <v>0</v>
+      </c>
+      <c r="G67" s="1">
+        <f t="shared" si="16"/>
+        <v>-123.86999999999999</v>
+      </c>
+      <c r="H67" s="6"/>
+      <c r="I67" s="5">
+        <v>0</v>
+      </c>
+      <c r="J67" s="5">
+        <f t="shared" si="17"/>
+        <v>-0.6</v>
+      </c>
+      <c r="K67" s="6"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1">
+        <f>B12*B65</f>
+        <v>2938.4169569999999</v>
+      </c>
+      <c r="C68" s="1">
+        <f>C12*B65</f>
+        <v>2899.5817905000004</v>
+      </c>
+      <c r="D68" s="1">
+        <f t="shared" ref="C68:D68" si="18">D12*D65</f>
+        <v>2045.7023262</v>
+      </c>
+      <c r="E68" s="6"/>
+      <c r="F68" s="1">
+        <f t="shared" ref="F61:F68" si="19">C68-B68</f>
+        <v>-38.835166499999559</v>
+      </c>
+      <c r="G68" s="1">
+        <f t="shared" ref="G61:G68" si="20">D68-B68</f>
+        <v>-892.7146307999999</v>
+      </c>
+      <c r="H68" s="6"/>
+      <c r="I68" s="5">
+        <f t="shared" si="15"/>
+        <v>-1.3216356653362302E-2</v>
+      </c>
+      <c r="J68" s="5">
+        <f t="shared" si="17"/>
+        <v>-0.30380801767201343</v>
+      </c>
+      <c r="K68" s="6"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" s="7"/>
+      <c r="B69" s="8"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="8"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="8"/>
+      <c r="J69" s="8"/>
+      <c r="K69" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="100">
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="I62:J62"/>
+    <mergeCell ref="I63:J63"/>
+    <mergeCell ref="I64:J64"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="I56:J56"/>
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="I59:J59"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="F1:G1"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="B10:D10"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
UPDATE: WIP - modify comparisons to include 3 datasets not 1.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_Red.xlsx
+++ b/FPGA_Performance_Comparison_Red.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC1CE82-BA68-2E4D-967C-7A116987A160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20F625B-F460-E242-B32D-FC7CCF8ADB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24100" windowHeight="26900" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="78">
   <si>
     <t>FPGA Implementation</t>
   </si>
@@ -252,6 +252,24 @@
   </si>
   <si>
     <t>Bit Manipulation Throttled</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Cotton</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Dino</t>
+  </si>
+  <si>
+    <t>Town</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
@@ -320,7 +338,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -359,8 +377,8 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -368,8 +386,14 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -706,7 +730,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45085A3-2BCA-FA4F-9A9B-A0D6975F9A68}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="50.83203125" style="3" customWidth="1"/>
@@ -716,15 +740,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
       <c r="F1" s="6"/>
       <c r="G1" s="15" t="s">
         <v>57</v>
@@ -740,7 +764,7 @@
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="17"/>
+      <c r="A2" s="14"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -865,10 +889,10 @@
       <c r="C5" s="1">
         <v>127.23</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="14">
         <v>201.53</v>
       </c>
-      <c r="E5" s="17"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="6"/>
       <c r="G5" s="1">
         <f>C5-B5</f>
@@ -923,10 +947,10 @@
       <c r="C7" s="1">
         <v>11790</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="14">
         <v>11914</v>
       </c>
-      <c r="E7" s="17"/>
+      <c r="E7" s="14"/>
       <c r="F7" s="6"/>
       <c r="G7" s="1">
         <f>C7-B7</f>
@@ -965,10 +989,10 @@
       <c r="C8" s="1">
         <v>27951</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="14">
         <v>30828</v>
       </c>
-      <c r="E8" s="17"/>
+      <c r="E8" s="14"/>
       <c r="F8" s="6"/>
       <c r="G8" s="1">
         <f>C8-B8</f>
@@ -1007,10 +1031,10 @@
       <c r="C9" s="1">
         <v>3199112</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="14">
         <v>3199112</v>
       </c>
-      <c r="E9" s="17"/>
+      <c r="E9" s="14"/>
       <c r="F9" s="6"/>
       <c r="G9" s="1">
         <f>C9-B9</f>
@@ -1049,10 +1073,10 @@
       <c r="C10" s="2">
         <v>12</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="14">
         <v>12</v>
       </c>
-      <c r="E10" s="17"/>
+      <c r="E10" s="14"/>
       <c r="F10" s="6"/>
       <c r="G10" s="1">
         <f>C10-B10</f>
@@ -1994,56 +2018,52 @@
       <c r="N32" s="6"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33" s="1">
-        <v>0.47430600000000001</v>
-      </c>
-      <c r="C33" s="15">
-        <v>2.0395829999999999</v>
-      </c>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
+      <c r="A33" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
       <c r="F33" s="6"/>
-      <c r="G33" s="15">
-        <f t="shared" ref="G33:G44" si="11">C33-B33</f>
-        <v>1.565277</v>
-      </c>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
+      <c r="G33" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="13">
-        <f>G33/B33</f>
-        <v>3.3001416806871515</v>
-      </c>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
+      <c r="K33" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
       <c r="N33" s="6"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="1">
-        <v>0.346667</v>
+        <v>0.47430600000000001</v>
       </c>
       <c r="C34" s="15">
-        <v>0.93874999999999997</v>
+        <v>2.0395829999999999</v>
       </c>
       <c r="D34" s="15"/>
       <c r="E34" s="15"/>
       <c r="F34" s="6"/>
       <c r="G34" s="15">
-        <f t="shared" si="11"/>
-        <v>0.59208299999999991</v>
+        <f t="shared" ref="G34:G45" si="11">C34-B34</f>
+        <v>1.565277</v>
       </c>
       <c r="H34" s="15"/>
       <c r="I34" s="15"/>
       <c r="J34" s="6"/>
       <c r="K34" s="13">
-        <f t="shared" ref="K34:K44" si="12">G34/B34</f>
-        <v>1.7079300885287607</v>
+        <f>G34/B34</f>
+        <v>3.3001416806871515</v>
       </c>
       <c r="L34" s="13"/>
       <c r="M34" s="13"/>
@@ -2051,26 +2071,27 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="1">
-        <v>0</v>
+        <v>0.346667</v>
       </c>
       <c r="C35" s="15">
-        <v>1</v>
+        <v>0.93874999999999997</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="15"/>
       <c r="F35" s="6"/>
       <c r="G35" s="15">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0.59208299999999991</v>
       </c>
       <c r="H35" s="15"/>
       <c r="I35" s="15"/>
       <c r="J35" s="6"/>
-      <c r="K35" s="13" t="s">
-        <v>56</v>
+      <c r="K35" s="13">
+        <f t="shared" ref="K35:K45" si="12">G35/B35</f>
+        <v>1.7079300885287607</v>
       </c>
       <c r="L35" s="13"/>
       <c r="M35" s="13"/>
@@ -2078,7 +2099,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="1">
         <v>0</v>
@@ -2105,27 +2126,26 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="C37" s="15">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D37" s="15"/>
       <c r="E37" s="15"/>
       <c r="F37" s="6"/>
       <c r="G37" s="15">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" s="15"/>
       <c r="I37" s="15"/>
       <c r="J37" s="6"/>
-      <c r="K37" s="13">
-        <f t="shared" si="12"/>
-        <v>-0.66666666666666663</v>
+      <c r="K37" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
@@ -2133,27 +2153,27 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" s="1">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="C38" s="15">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
       <c r="F38" s="6"/>
       <c r="G38" s="15">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H38" s="15"/>
       <c r="I38" s="15"/>
       <c r="J38" s="6"/>
       <c r="K38" s="13">
         <f t="shared" si="12"/>
-        <v>6</v>
+        <v>-0.66666666666666663</v>
       </c>
       <c r="L38" s="13"/>
       <c r="M38" s="13"/>
@@ -2161,27 +2181,27 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="1">
-        <v>7.6160420000000002</v>
+        <v>1</v>
       </c>
       <c r="C39" s="15">
-        <v>7.1617360000000003</v>
+        <v>7</v>
       </c>
       <c r="D39" s="15"/>
       <c r="E39" s="15"/>
       <c r="F39" s="6"/>
       <c r="G39" s="15">
         <f t="shared" si="11"/>
-        <v>-0.45430599999999988</v>
+        <v>6</v>
       </c>
       <c r="H39" s="15"/>
       <c r="I39" s="15"/>
       <c r="J39" s="6"/>
       <c r="K39" s="13">
         <f t="shared" si="12"/>
-        <v>-5.9651194150452412E-2</v>
+        <v>6</v>
       </c>
       <c r="L39" s="13"/>
       <c r="M39" s="13"/>
@@ -2189,27 +2209,27 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" s="1">
-        <v>8</v>
+        <v>7.6160420000000002</v>
       </c>
       <c r="C40" s="15">
-        <v>7</v>
+        <v>7.1617360000000003</v>
       </c>
       <c r="D40" s="15"/>
       <c r="E40" s="15"/>
       <c r="F40" s="6"/>
       <c r="G40" s="15">
         <f t="shared" si="11"/>
-        <v>-1</v>
+        <v>-0.45430599999999988</v>
       </c>
       <c r="H40" s="15"/>
       <c r="I40" s="15"/>
       <c r="J40" s="6"/>
       <c r="K40" s="13">
         <f t="shared" si="12"/>
-        <v>-0.125</v>
+        <v>-5.9651194150452412E-2</v>
       </c>
       <c r="L40" s="13"/>
       <c r="M40" s="13"/>
@@ -2217,27 +2237,27 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" s="1">
         <v>8</v>
       </c>
       <c r="C41" s="15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D41" s="15"/>
       <c r="E41" s="15"/>
       <c r="F41" s="6"/>
       <c r="G41" s="15">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H41" s="15"/>
       <c r="I41" s="15"/>
       <c r="J41" s="6"/>
       <c r="K41" s="13">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>-0.125</v>
       </c>
       <c r="L41" s="13"/>
       <c r="M41" s="13"/>
@@ -2245,27 +2265,27 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C42" s="15">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D42" s="15"/>
       <c r="E42" s="15"/>
       <c r="F42" s="6"/>
       <c r="G42" s="15">
         <f t="shared" si="11"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H42" s="15"/>
       <c r="I42" s="15"/>
       <c r="J42" s="6"/>
       <c r="K42" s="13">
         <f t="shared" si="12"/>
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="L42" s="13"/>
       <c r="M42" s="13"/>
@@ -2273,27 +2293,27 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="1">
-        <v>10234</v>
+        <v>5</v>
       </c>
       <c r="C43" s="15">
-        <v>6033</v>
+        <v>4</v>
       </c>
       <c r="D43" s="15"/>
       <c r="E43" s="15"/>
       <c r="F43" s="6"/>
       <c r="G43" s="15">
         <f t="shared" si="11"/>
-        <v>-4201</v>
+        <v>-1</v>
       </c>
       <c r="H43" s="15"/>
       <c r="I43" s="15"/>
       <c r="J43" s="6"/>
       <c r="K43" s="13">
         <f t="shared" si="12"/>
-        <v>-0.41049443033027166</v>
+        <v>-0.2</v>
       </c>
       <c r="L43" s="13"/>
       <c r="M43" s="13"/>
@@ -2301,127 +2321,123 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44" s="5">
-        <v>0.71069444000000004</v>
-      </c>
-      <c r="C44" s="16">
-        <v>0.41895832999999999</v>
-      </c>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
+        <v>42</v>
+      </c>
+      <c r="B44" s="1">
+        <v>10234</v>
+      </c>
+      <c r="C44" s="15">
+        <v>6033</v>
+      </c>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
       <c r="F44" s="6"/>
       <c r="G44" s="15">
         <f t="shared" si="11"/>
-        <v>-0.29173611000000005</v>
+        <v>-4201</v>
       </c>
       <c r="H44" s="15"/>
       <c r="I44" s="15"/>
       <c r="J44" s="6"/>
       <c r="K44" s="13">
         <f t="shared" si="12"/>
-        <v>-0.41049443133394997</v>
+        <v>-0.41049443033027166</v>
       </c>
       <c r="L44" s="13"/>
       <c r="M44" s="13"/>
       <c r="N44" s="6"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A45" s="7"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="8"/>
+      <c r="A45" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="5">
+        <v>0.71069444000000004</v>
+      </c>
+      <c r="C45" s="16">
+        <v>0.41895832999999999</v>
+      </c>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
       <c r="F45" s="6"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
+      <c r="G45" s="15">
+        <f t="shared" si="11"/>
+        <v>-0.29173611000000005</v>
+      </c>
+      <c r="H45" s="15"/>
+      <c r="I45" s="15"/>
       <c r="J45" s="6"/>
-      <c r="K45" s="8"/>
-      <c r="L45" s="8"/>
-      <c r="M45" s="8"/>
+      <c r="K45" s="13">
+        <f t="shared" si="12"/>
+        <v>-0.41049443133394997</v>
+      </c>
+      <c r="L45" s="13"/>
+      <c r="M45" s="13"/>
       <c r="N45" s="6"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" s="1">
-        <v>4.131875</v>
-      </c>
-      <c r="C46" s="15">
-        <v>3.605556</v>
-      </c>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
+      <c r="A46" s="7"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="8"/>
       <c r="F46" s="6"/>
-      <c r="G46" s="15">
-        <f t="shared" ref="G46:G57" si="13">C46-B46</f>
-        <v>-0.52631899999999998</v>
-      </c>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="8"/>
       <c r="J46" s="6"/>
-      <c r="K46" s="13">
-        <f>G46/B46</f>
-        <v>-0.12738018454091665</v>
-      </c>
-      <c r="L46" s="13"/>
-      <c r="M46" s="13"/>
+      <c r="K46" s="8"/>
+      <c r="L46" s="8"/>
+      <c r="M46" s="8"/>
       <c r="N46" s="6"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B47" s="1">
-        <v>1.9239580000000001</v>
-      </c>
-      <c r="C47" s="15">
-        <v>1.838889</v>
-      </c>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
+      <c r="A47" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
       <c r="F47" s="6"/>
-      <c r="G47" s="15">
-        <f t="shared" si="13"/>
-        <v>-8.5069000000000061E-2</v>
-      </c>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
+      <c r="G47" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H47" s="19"/>
+      <c r="I47" s="19"/>
       <c r="J47" s="6"/>
-      <c r="K47" s="13">
-        <f t="shared" ref="K47:K57" si="14">G47/B47</f>
-        <v>-4.4215622170546372E-2</v>
-      </c>
-      <c r="L47" s="13"/>
-      <c r="M47" s="13"/>
+      <c r="K47" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L47" s="19"/>
+      <c r="M47" s="19"/>
       <c r="N47" s="6"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B48" s="1">
-        <v>2</v>
+        <v>4.131875</v>
       </c>
       <c r="C48" s="15">
-        <v>2</v>
+        <v>3.605556</v>
       </c>
       <c r="D48" s="15"/>
       <c r="E48" s="15"/>
       <c r="F48" s="6"/>
       <c r="G48" s="15">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <f t="shared" ref="G48:G59" si="13">C48-B48</f>
+        <v>-0.52631899999999998</v>
       </c>
       <c r="H48" s="15"/>
       <c r="I48" s="15"/>
       <c r="J48" s="6"/>
       <c r="K48" s="13">
-        <f t="shared" si="14"/>
-        <v>0</v>
+        <f>G48/B48</f>
+        <v>-0.12738018454091665</v>
       </c>
       <c r="L48" s="13"/>
       <c r="M48" s="13"/>
@@ -2429,27 +2445,27 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B49" s="1">
-        <v>-2</v>
+        <v>1.9239580000000001</v>
       </c>
       <c r="C49" s="15">
-        <v>-2</v>
+        <v>1.838889</v>
       </c>
       <c r="D49" s="15"/>
       <c r="E49" s="15"/>
       <c r="F49" s="6"/>
       <c r="G49" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-8.5069000000000061E-2</v>
       </c>
       <c r="H49" s="15"/>
       <c r="I49" s="15"/>
       <c r="J49" s="6"/>
       <c r="K49" s="13">
-        <f t="shared" si="14"/>
-        <v>0</v>
+        <f t="shared" ref="K49:K59" si="14">G49/B49</f>
+        <v>-4.4215622170546372E-2</v>
       </c>
       <c r="L49" s="13"/>
       <c r="M49" s="13"/>
@@ -2457,13 +2473,13 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B50" s="1">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="C50" s="15">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="D50" s="15"/>
       <c r="E50" s="15"/>
@@ -2485,27 +2501,27 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B51" s="1">
-        <v>19</v>
+        <v>-2</v>
       </c>
       <c r="C51" s="15">
-        <v>3</v>
+        <v>-2</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="15"/>
       <c r="F51" s="6"/>
       <c r="G51" s="15">
         <f t="shared" si="13"/>
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="H51" s="15"/>
       <c r="I51" s="15"/>
       <c r="J51" s="6"/>
       <c r="K51" s="13">
         <f t="shared" si="14"/>
-        <v>-0.84210526315789469</v>
+        <v>0</v>
       </c>
       <c r="L51" s="13"/>
       <c r="M51" s="13"/>
@@ -2513,27 +2529,27 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B52" s="1">
-        <v>6.8117359999999998</v>
+        <v>-3</v>
       </c>
       <c r="C52" s="15">
-        <v>6.8386810000000002</v>
+        <v>-3</v>
       </c>
       <c r="D52" s="15"/>
       <c r="E52" s="15"/>
       <c r="F52" s="6"/>
       <c r="G52" s="15">
         <f t="shared" si="13"/>
-        <v>2.6945000000000441E-2</v>
+        <v>0</v>
       </c>
       <c r="H52" s="15"/>
       <c r="I52" s="15"/>
       <c r="J52" s="6"/>
       <c r="K52" s="13">
         <f t="shared" si="14"/>
-        <v>3.9556729738205419E-3</v>
+        <v>0</v>
       </c>
       <c r="L52" s="13"/>
       <c r="M52" s="13"/>
@@ -2541,27 +2557,27 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B53" s="1">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C53" s="15">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="15"/>
       <c r="F53" s="6"/>
       <c r="G53" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="H53" s="15"/>
       <c r="I53" s="15"/>
       <c r="J53" s="6"/>
       <c r="K53" s="13">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>-0.84210526315789469</v>
       </c>
       <c r="L53" s="13"/>
       <c r="M53" s="13"/>
@@ -2569,27 +2585,27 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B54" s="1">
-        <v>8</v>
+        <v>6.8117359999999998</v>
       </c>
       <c r="C54" s="15">
-        <v>8</v>
+        <v>6.8386810000000002</v>
       </c>
       <c r="D54" s="15"/>
       <c r="E54" s="15"/>
       <c r="F54" s="6"/>
       <c r="G54" s="15">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.6945000000000441E-2</v>
       </c>
       <c r="H54" s="15"/>
       <c r="I54" s="15"/>
       <c r="J54" s="6"/>
       <c r="K54" s="13">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>3.9556729738205419E-3</v>
       </c>
       <c r="L54" s="13"/>
       <c r="M54" s="13"/>
@@ -2597,27 +2613,27 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B55" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C55" s="15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D55" s="15"/>
       <c r="E55" s="15"/>
       <c r="F55" s="6"/>
       <c r="G55" s="15">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H55" s="15"/>
       <c r="I55" s="15"/>
       <c r="J55" s="6"/>
       <c r="K55" s="13">
         <f t="shared" si="14"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="L55" s="13"/>
       <c r="M55" s="13"/>
@@ -2625,27 +2641,27 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B56" s="1">
-        <v>195</v>
+        <v>8</v>
       </c>
       <c r="C56" s="15">
-        <v>274</v>
+        <v>8</v>
       </c>
       <c r="D56" s="15"/>
       <c r="E56" s="15"/>
       <c r="F56" s="6"/>
       <c r="G56" s="15">
         <f t="shared" si="13"/>
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="H56" s="15"/>
       <c r="I56" s="15"/>
       <c r="J56" s="6"/>
       <c r="K56" s="13">
         <f t="shared" si="14"/>
-        <v>0.40512820512820513</v>
+        <v>0</v>
       </c>
       <c r="L56" s="13"/>
       <c r="M56" s="13"/>
@@ -2653,142 +2669,151 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B57" s="5">
-        <v>1.354167E-2</v>
-      </c>
-      <c r="C57" s="13">
-        <v>1.9027780000000001E-2</v>
-      </c>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
+        <v>53</v>
+      </c>
+      <c r="B57" s="1">
+        <v>4</v>
+      </c>
+      <c r="C57" s="15">
+        <v>5</v>
+      </c>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
       <c r="F57" s="6"/>
       <c r="G57" s="15">
         <f t="shared" si="13"/>
-        <v>5.4861100000000006E-3</v>
+        <v>1</v>
       </c>
       <c r="H57" s="15"/>
       <c r="I57" s="15"/>
       <c r="J57" s="6"/>
       <c r="K57" s="13">
         <f t="shared" si="14"/>
-        <v>0.405128023353102</v>
+        <v>0.25</v>
       </c>
       <c r="L57" s="13"/>
       <c r="M57" s="13"/>
       <c r="N57" s="6"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A58" s="7"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="8"/>
+      <c r="A58" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B58" s="1">
+        <v>195</v>
+      </c>
+      <c r="C58" s="15">
+        <v>274</v>
+      </c>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
       <c r="F58" s="6"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="8"/>
-      <c r="I58" s="8"/>
+      <c r="G58" s="15">
+        <f t="shared" si="13"/>
+        <v>79</v>
+      </c>
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
       <c r="J58" s="6"/>
-      <c r="K58" s="8"/>
-      <c r="L58" s="8"/>
-      <c r="M58" s="8"/>
+      <c r="K58" s="13">
+        <f t="shared" si="14"/>
+        <v>0.40512820512820513</v>
+      </c>
+      <c r="L58" s="13"/>
+      <c r="M58" s="13"/>
       <c r="N58" s="6"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B59" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
+        <v>55</v>
+      </c>
+      <c r="B59" s="5">
+        <v>1.354167E-2</v>
+      </c>
+      <c r="C59" s="13">
+        <v>1.9027780000000001E-2</v>
+      </c>
+      <c r="D59" s="13"/>
+      <c r="E59" s="13"/>
       <c r="F59" s="6"/>
       <c r="G59" s="15">
-        <v>0</v>
+        <f t="shared" si="13"/>
+        <v>5.4861100000000006E-3</v>
       </c>
       <c r="H59" s="15"/>
       <c r="I59" s="15"/>
       <c r="J59" s="6"/>
-      <c r="K59" s="14">
-        <v>0</v>
-      </c>
-      <c r="L59" s="14"/>
-      <c r="M59" s="14"/>
+      <c r="K59" s="13">
+        <f t="shared" si="14"/>
+        <v>0.405128023353102</v>
+      </c>
+      <c r="L59" s="13"/>
+      <c r="M59" s="13"/>
       <c r="N59" s="6"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B60" s="15">
-        <v>1</v>
-      </c>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
+      <c r="A60" s="7"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="8"/>
       <c r="F60" s="6"/>
-      <c r="G60" s="15">
-        <v>0</v>
-      </c>
-      <c r="H60" s="15"/>
-      <c r="I60" s="15"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8"/>
       <c r="J60" s="6"/>
-      <c r="K60" s="13">
-        <f>G60/B60</f>
-        <v>0</v>
-      </c>
-      <c r="L60" s="13"/>
-      <c r="M60" s="13"/>
+      <c r="K60" s="8"/>
+      <c r="L60" s="8"/>
+      <c r="M60" s="8"/>
       <c r="N60" s="6"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B61" s="15">
-        <v>278529</v>
-      </c>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
+      <c r="A61" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B61" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C61" s="19"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
       <c r="F61" s="6"/>
-      <c r="G61" s="15">
-        <v>0</v>
-      </c>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
+      <c r="G61" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H61" s="19"/>
+      <c r="I61" s="19"/>
       <c r="J61" s="6"/>
-      <c r="K61" s="13">
-        <f>G61/B61</f>
-        <v>0</v>
-      </c>
-      <c r="L61" s="13"/>
-      <c r="M61" s="13"/>
+      <c r="K61" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L61" s="19"/>
+      <c r="M61" s="19"/>
       <c r="N61" s="6"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="15">
-        <v>279694</v>
-      </c>
-      <c r="C62" s="15"/>
+        <v>32</v>
+      </c>
+      <c r="B62" s="1">
+        <v>0.47430600000000001</v>
+      </c>
+      <c r="C62" s="15">
+        <v>3.1540180000000002</v>
+      </c>
       <c r="D62" s="15"/>
       <c r="E62" s="15"/>
       <c r="F62" s="6"/>
       <c r="G62" s="15">
-        <v>0</v>
+        <f t="shared" ref="G62:G73" si="15">C62-B62</f>
+        <v>2.6797120000000003</v>
       </c>
       <c r="H62" s="15"/>
       <c r="I62" s="15"/>
       <c r="J62" s="6"/>
       <c r="K62" s="13">
         <f>G62/B62</f>
-        <v>0</v>
+        <v>5.649753534637977</v>
       </c>
       <c r="L62" s="13"/>
       <c r="M62" s="13"/>
@@ -2796,24 +2821,27 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B63" s="15">
-        <v>295045</v>
-      </c>
-      <c r="C63" s="15"/>
+        <v>33</v>
+      </c>
+      <c r="B63" s="1">
+        <v>0.346667</v>
+      </c>
+      <c r="C63" s="15">
+        <v>1.2675380000000001</v>
+      </c>
       <c r="D63" s="15"/>
       <c r="E63" s="15"/>
       <c r="F63" s="6"/>
       <c r="G63" s="15">
-        <v>0</v>
+        <f t="shared" si="15"/>
+        <v>0.920871</v>
       </c>
       <c r="H63" s="15"/>
       <c r="I63" s="15"/>
       <c r="J63" s="6"/>
       <c r="K63" s="13">
-        <f>G63/B63</f>
-        <v>0</v>
+        <f t="shared" ref="K63:K73" si="16">G63/B63</f>
+        <v>2.6563560996575966</v>
       </c>
       <c r="L63" s="13"/>
       <c r="M63" s="13"/>
@@ -2821,25 +2849,26 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B64" s="15">
-        <f>B63-B60</f>
-        <v>295044</v>
-      </c>
-      <c r="C64" s="15"/>
+        <v>34</v>
+      </c>
+      <c r="B64" s="1">
+        <v>0</v>
+      </c>
+      <c r="C64" s="15">
+        <v>1</v>
+      </c>
       <c r="D64" s="15"/>
       <c r="E64" s="15"/>
       <c r="F64" s="6"/>
       <c r="G64" s="15">
-        <v>0</v>
+        <f t="shared" si="15"/>
+        <v>1</v>
       </c>
       <c r="H64" s="15"/>
       <c r="I64" s="15"/>
       <c r="J64" s="6"/>
-      <c r="K64" s="13">
-        <f>G64/B64</f>
-        <v>0</v>
+      <c r="K64" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
@@ -2847,58 +2876,53 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B65" s="15">
-        <f>B64/(B3*10^3)</f>
-        <v>3.6880500000000001</v>
-      </c>
-      <c r="C65" s="15"/>
+        <v>35</v>
+      </c>
+      <c r="B65" s="1">
+        <v>0</v>
+      </c>
+      <c r="C65" s="15">
+        <v>1</v>
+      </c>
       <c r="D65" s="15"/>
-      <c r="E65" s="1">
-        <f>B64/(E3*10^3)</f>
-        <v>1.47522</v>
-      </c>
+      <c r="E65" s="15"/>
       <c r="F65" s="6"/>
       <c r="G65" s="15">
-        <v>0</v>
+        <f t="shared" si="15"/>
+        <v>1</v>
       </c>
       <c r="H65" s="15"/>
-      <c r="I65" s="1">
-        <f>E65-B65</f>
-        <v>-2.2128300000000003</v>
-      </c>
+      <c r="I65" s="15"/>
       <c r="J65" s="6"/>
-      <c r="K65" s="13">
-        <v>0</v>
+      <c r="K65" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="L65" s="13"/>
-      <c r="M65" s="5">
-        <f>I65/B65</f>
-        <v>-0.60000000000000009</v>
-      </c>
+      <c r="M65" s="13"/>
       <c r="N65" s="6"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66" s="15">
-        <f>B63-B61</f>
-        <v>16516</v>
-      </c>
-      <c r="C66" s="15"/>
+        <v>36</v>
+      </c>
+      <c r="B66" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C66" s="15">
+        <v>-3</v>
+      </c>
       <c r="D66" s="15"/>
       <c r="E66" s="15"/>
       <c r="F66" s="6"/>
       <c r="G66" s="15">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="H66" s="15"/>
       <c r="I66" s="15"/>
       <c r="J66" s="6"/>
       <c r="K66" s="13">
-        <f>G66/B66</f>
+        <f t="shared" ref="K66:K76" si="17">G66/B66</f>
         <v>0</v>
       </c>
       <c r="L66" s="13"/>
@@ -2907,184 +2931,2713 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B67" s="15">
-        <f>B66/B3</f>
-        <v>206.45</v>
-      </c>
-      <c r="C67" s="15"/>
+        <v>37</v>
+      </c>
+      <c r="B67" s="1">
+        <v>1</v>
+      </c>
+      <c r="C67" s="15">
+        <v>6</v>
+      </c>
       <c r="D67" s="15"/>
-      <c r="E67" s="1">
-        <f>B66/E3</f>
-        <v>82.58</v>
-      </c>
+      <c r="E67" s="15"/>
       <c r="F67" s="6"/>
       <c r="G67" s="15">
-        <v>0</v>
+        <f t="shared" si="15"/>
+        <v>5</v>
       </c>
       <c r="H67" s="15"/>
-      <c r="I67" s="1">
-        <f>E67-B67</f>
-        <v>-123.86999999999999</v>
-      </c>
+      <c r="I67" s="15"/>
       <c r="J67" s="6"/>
       <c r="K67" s="13">
-        <v>0</v>
+        <f t="shared" si="17"/>
+        <v>5</v>
       </c>
       <c r="L67" s="13"/>
-      <c r="M67" s="5">
-        <f>I67/B67</f>
-        <v>-0.6</v>
-      </c>
+      <c r="M67" s="13"/>
       <c r="N67" s="6"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="B68" s="1">
-        <f>B12*B65</f>
-        <v>2938.4169569999999</v>
-      </c>
-      <c r="C68" s="1">
-        <f>C12*B65</f>
-        <v>2899.5817905000004</v>
-      </c>
-      <c r="D68" s="11">
-        <f>D12*B65</f>
-        <v>2987.4311414999997</v>
-      </c>
-      <c r="E68" s="1">
-        <f t="shared" ref="E68" si="15">E12*E65</f>
-        <v>2045.7023262</v>
-      </c>
+        <v>7.6160420000000002</v>
+      </c>
+      <c r="C68" s="15">
+        <v>6.9878830000000001</v>
+      </c>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
       <c r="F68" s="6"/>
-      <c r="G68" s="1">
-        <f>C68-B68</f>
-        <v>-38.835166499999559</v>
-      </c>
-      <c r="H68" s="1">
-        <f>D68-B68</f>
-        <v>49.014184499999828</v>
-      </c>
-      <c r="I68" s="1">
-        <f>E68-B68</f>
-        <v>-892.7146307999999</v>
-      </c>
+      <c r="G68" s="15">
+        <f t="shared" si="15"/>
+        <v>-0.62815900000000013</v>
+      </c>
+      <c r="H68" s="15"/>
+      <c r="I68" s="15"/>
       <c r="J68" s="6"/>
-      <c r="K68" s="5">
-        <f>G68/B68</f>
-        <v>-1.3216356653362302E-2</v>
-      </c>
-      <c r="L68" s="5">
-        <f>H68/B68</f>
-        <v>1.6680472927178194E-2</v>
-      </c>
-      <c r="M68" s="5"/>
+      <c r="K68" s="13">
+        <f t="shared" si="17"/>
+        <v>-8.2478405449969955E-2</v>
+      </c>
+      <c r="L68" s="13"/>
+      <c r="M68" s="13"/>
       <c r="N68" s="6"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B69" s="15">
-        <f>1/(B65/1000)</f>
-        <v>271.1459985629262</v>
-      </c>
-      <c r="C69" s="15"/>
+        <v>39</v>
+      </c>
+      <c r="B69" s="1">
+        <v>8</v>
+      </c>
+      <c r="C69" s="15">
+        <v>7</v>
+      </c>
       <c r="D69" s="15"/>
-      <c r="E69" s="1">
-        <f>1/(E65/1000)</f>
-        <v>677.86499640731552</v>
-      </c>
+      <c r="E69" s="15"/>
       <c r="F69" s="6"/>
       <c r="G69" s="15">
-        <v>0</v>
+        <f t="shared" si="15"/>
+        <v>-1</v>
       </c>
       <c r="H69" s="15"/>
-      <c r="I69" s="1">
-        <f>E69-B69</f>
-        <v>406.71899784438932</v>
-      </c>
+      <c r="I69" s="15"/>
       <c r="J69" s="6"/>
       <c r="K69" s="13">
-        <v>0</v>
+        <f t="shared" si="17"/>
+        <v>-0.125</v>
       </c>
       <c r="L69" s="13"/>
-      <c r="M69" s="5">
-        <f>I69/B69</f>
+      <c r="M69" s="13"/>
+      <c r="N69" s="6"/>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B70" s="1">
+        <v>8</v>
+      </c>
+      <c r="C70" s="15">
+        <v>8</v>
+      </c>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="15">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="H70" s="15"/>
+      <c r="I70" s="15"/>
+      <c r="J70" s="6"/>
+      <c r="K70" s="13">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="L70" s="13"/>
+      <c r="M70" s="13"/>
+      <c r="N70" s="6"/>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B71" s="1">
+        <v>5</v>
+      </c>
+      <c r="C71" s="15">
+        <v>5</v>
+      </c>
+      <c r="D71" s="15"/>
+      <c r="E71" s="15"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="15">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="H71" s="15"/>
+      <c r="I71" s="15"/>
+      <c r="J71" s="6"/>
+      <c r="K71" s="13">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="L71" s="13"/>
+      <c r="M71" s="13"/>
+      <c r="N71" s="6"/>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B72" s="1">
+        <v>10234</v>
+      </c>
+      <c r="C72" s="15">
+        <v>902</v>
+      </c>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="15">
+        <f t="shared" si="15"/>
+        <v>-9332</v>
+      </c>
+      <c r="H72" s="15"/>
+      <c r="I72" s="15"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="13">
+        <f t="shared" si="17"/>
+        <v>-0.91186241938635915</v>
+      </c>
+      <c r="L72" s="13"/>
+      <c r="M72" s="13"/>
+      <c r="N72" s="6"/>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B73" s="5">
+        <v>0.71069444000000004</v>
+      </c>
+      <c r="C73" s="16">
+        <v>0.41895832999999999</v>
+      </c>
+      <c r="D73" s="16"/>
+      <c r="E73" s="16"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="15">
+        <f t="shared" si="15"/>
+        <v>-0.29173611000000005</v>
+      </c>
+      <c r="H73" s="15"/>
+      <c r="I73" s="15"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="13">
+        <f t="shared" si="17"/>
+        <v>-0.41049443133394997</v>
+      </c>
+      <c r="L73" s="13"/>
+      <c r="M73" s="13"/>
+      <c r="N73" s="6"/>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A74" s="7"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="6"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="8"/>
+      <c r="I74" s="8"/>
+      <c r="J74" s="6"/>
+      <c r="K74" s="8"/>
+      <c r="L74" s="8"/>
+      <c r="M74" s="8"/>
+      <c r="N74" s="6"/>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A75" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B75" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C75" s="19"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="19"/>
+      <c r="F75" s="6"/>
+      <c r="G75" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H75" s="19"/>
+      <c r="I75" s="19"/>
+      <c r="J75" s="6"/>
+      <c r="K75" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L75" s="19"/>
+      <c r="M75" s="19"/>
+      <c r="N75" s="6"/>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B76" s="1">
+        <v>4.131875</v>
+      </c>
+      <c r="C76" s="15">
+        <v>3.605556</v>
+      </c>
+      <c r="D76" s="15"/>
+      <c r="E76" s="15"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="15">
+        <f t="shared" ref="G76:G87" si="18">C76-B76</f>
+        <v>-0.52631899999999998</v>
+      </c>
+      <c r="H76" s="15"/>
+      <c r="I76" s="15"/>
+      <c r="J76" s="6"/>
+      <c r="K76" s="13">
+        <f>G76/B76</f>
+        <v>-0.12738018454091665</v>
+      </c>
+      <c r="L76" s="13"/>
+      <c r="M76" s="13"/>
+      <c r="N76" s="6"/>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B77" s="1">
+        <v>1.9239580000000001</v>
+      </c>
+      <c r="C77" s="15">
+        <v>1.838889</v>
+      </c>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="15">
+        <f t="shared" si="18"/>
+        <v>-8.5069000000000061E-2</v>
+      </c>
+      <c r="H77" s="15"/>
+      <c r="I77" s="15"/>
+      <c r="J77" s="6"/>
+      <c r="K77" s="13">
+        <f t="shared" ref="K77:K87" si="19">G77/B77</f>
+        <v>-4.4215622170546372E-2</v>
+      </c>
+      <c r="L77" s="13"/>
+      <c r="M77" s="13"/>
+      <c r="N77" s="6"/>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B78" s="1">
+        <v>2</v>
+      </c>
+      <c r="C78" s="15">
+        <v>2</v>
+      </c>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="15">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H78" s="15"/>
+      <c r="I78" s="15"/>
+      <c r="J78" s="6"/>
+      <c r="K78" s="13">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L78" s="13"/>
+      <c r="M78" s="13"/>
+      <c r="N78" s="6"/>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B79" s="1">
+        <v>-2</v>
+      </c>
+      <c r="C79" s="15">
+        <v>-2</v>
+      </c>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15"/>
+      <c r="F79" s="6"/>
+      <c r="G79" s="15">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H79" s="15"/>
+      <c r="I79" s="15"/>
+      <c r="J79" s="6"/>
+      <c r="K79" s="13">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L79" s="13"/>
+      <c r="M79" s="13"/>
+      <c r="N79" s="6"/>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B80" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C80" s="15">
+        <v>-3</v>
+      </c>
+      <c r="D80" s="15"/>
+      <c r="E80" s="15"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="15">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H80" s="15"/>
+      <c r="I80" s="15"/>
+      <c r="J80" s="6"/>
+      <c r="K80" s="13">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L80" s="13"/>
+      <c r="M80" s="13"/>
+      <c r="N80" s="6"/>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B81" s="1">
+        <v>19</v>
+      </c>
+      <c r="C81" s="15">
+        <v>3</v>
+      </c>
+      <c r="D81" s="15"/>
+      <c r="E81" s="15"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="15">
+        <f t="shared" si="18"/>
+        <v>-16</v>
+      </c>
+      <c r="H81" s="15"/>
+      <c r="I81" s="15"/>
+      <c r="J81" s="6"/>
+      <c r="K81" s="13">
+        <f t="shared" si="19"/>
+        <v>-0.84210526315789469</v>
+      </c>
+      <c r="L81" s="13"/>
+      <c r="M81" s="13"/>
+      <c r="N81" s="6"/>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A82" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B82" s="1">
+        <v>6.8117359999999998</v>
+      </c>
+      <c r="C82" s="15">
+        <v>6.8386810000000002</v>
+      </c>
+      <c r="D82" s="15"/>
+      <c r="E82" s="15"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="15">
+        <f t="shared" si="18"/>
+        <v>2.6945000000000441E-2</v>
+      </c>
+      <c r="H82" s="15"/>
+      <c r="I82" s="15"/>
+      <c r="J82" s="6"/>
+      <c r="K82" s="13">
+        <f t="shared" si="19"/>
+        <v>3.9556729738205419E-3</v>
+      </c>
+      <c r="L82" s="13"/>
+      <c r="M82" s="13"/>
+      <c r="N82" s="6"/>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B83" s="1">
+        <v>7</v>
+      </c>
+      <c r="C83" s="15">
+        <v>7</v>
+      </c>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="6"/>
+      <c r="G83" s="15">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H83" s="15"/>
+      <c r="I83" s="15"/>
+      <c r="J83" s="6"/>
+      <c r="K83" s="13">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L83" s="13"/>
+      <c r="M83" s="13"/>
+      <c r="N83" s="6"/>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84" s="1">
+        <v>8</v>
+      </c>
+      <c r="C84" s="15">
+        <v>8</v>
+      </c>
+      <c r="D84" s="15"/>
+      <c r="E84" s="15"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="15">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H84" s="15"/>
+      <c r="I84" s="15"/>
+      <c r="J84" s="6"/>
+      <c r="K84" s="13">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L84" s="13"/>
+      <c r="M84" s="13"/>
+      <c r="N84" s="6"/>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B85" s="1">
+        <v>4</v>
+      </c>
+      <c r="C85" s="15">
+        <v>5</v>
+      </c>
+      <c r="D85" s="15"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="15">
+        <f t="shared" si="18"/>
+        <v>1</v>
+      </c>
+      <c r="H85" s="15"/>
+      <c r="I85" s="15"/>
+      <c r="J85" s="6"/>
+      <c r="K85" s="13">
+        <f t="shared" si="19"/>
+        <v>0.25</v>
+      </c>
+      <c r="L85" s="13"/>
+      <c r="M85" s="13"/>
+      <c r="N85" s="6"/>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B86" s="1">
+        <v>195</v>
+      </c>
+      <c r="C86" s="15">
+        <v>274</v>
+      </c>
+      <c r="D86" s="15"/>
+      <c r="E86" s="15"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="15">
+        <f t="shared" si="18"/>
+        <v>79</v>
+      </c>
+      <c r="H86" s="15"/>
+      <c r="I86" s="15"/>
+      <c r="J86" s="6"/>
+      <c r="K86" s="13">
+        <f t="shared" si="19"/>
+        <v>0.40512820512820513</v>
+      </c>
+      <c r="L86" s="13"/>
+      <c r="M86" s="13"/>
+      <c r="N86" s="6"/>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B87" s="5">
+        <v>1.354167E-2</v>
+      </c>
+      <c r="C87" s="13">
+        <v>1.9027780000000001E-2</v>
+      </c>
+      <c r="D87" s="13"/>
+      <c r="E87" s="13"/>
+      <c r="F87" s="6"/>
+      <c r="G87" s="15">
+        <f t="shared" si="18"/>
+        <v>5.4861100000000006E-3</v>
+      </c>
+      <c r="H87" s="15"/>
+      <c r="I87" s="15"/>
+      <c r="J87" s="6"/>
+      <c r="K87" s="13">
+        <f t="shared" si="19"/>
+        <v>0.405128023353102</v>
+      </c>
+      <c r="L87" s="13"/>
+      <c r="M87" s="13"/>
+      <c r="N87" s="6"/>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A88" s="7"/>
+      <c r="B88" s="8"/>
+      <c r="C88" s="8"/>
+      <c r="D88" s="12"/>
+      <c r="E88" s="8"/>
+      <c r="F88" s="6"/>
+      <c r="G88" s="8"/>
+      <c r="H88" s="8"/>
+      <c r="I88" s="8"/>
+      <c r="J88" s="6"/>
+      <c r="K88" s="8"/>
+      <c r="L88" s="8"/>
+      <c r="M88" s="8"/>
+      <c r="N88" s="6"/>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A89" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B89" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C89" s="19"/>
+      <c r="D89" s="19"/>
+      <c r="E89" s="19"/>
+      <c r="F89" s="6"/>
+      <c r="G89" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H89" s="19"/>
+      <c r="I89" s="19"/>
+      <c r="J89" s="6"/>
+      <c r="K89" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L89" s="19"/>
+      <c r="M89" s="19"/>
+      <c r="N89" s="6"/>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A90" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" s="1">
+        <v>0.47430600000000001</v>
+      </c>
+      <c r="C90" s="15">
+        <v>2.0395829999999999</v>
+      </c>
+      <c r="D90" s="15"/>
+      <c r="E90" s="15"/>
+      <c r="F90" s="6"/>
+      <c r="G90" s="15">
+        <f t="shared" ref="G90:G101" si="20">C90-B90</f>
+        <v>1.565277</v>
+      </c>
+      <c r="H90" s="15"/>
+      <c r="I90" s="15"/>
+      <c r="J90" s="6"/>
+      <c r="K90" s="13">
+        <f>G90/B90</f>
+        <v>3.3001416806871515</v>
+      </c>
+      <c r="L90" s="13"/>
+      <c r="M90" s="13"/>
+      <c r="N90" s="6"/>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A91" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B91" s="1">
+        <v>0.346667</v>
+      </c>
+      <c r="C91" s="15">
+        <v>0.93874999999999997</v>
+      </c>
+      <c r="D91" s="15"/>
+      <c r="E91" s="15"/>
+      <c r="F91" s="6"/>
+      <c r="G91" s="15">
+        <f t="shared" si="20"/>
+        <v>0.59208299999999991</v>
+      </c>
+      <c r="H91" s="15"/>
+      <c r="I91" s="15"/>
+      <c r="J91" s="6"/>
+      <c r="K91" s="13">
+        <f t="shared" ref="K91:K101" si="21">G91/B91</f>
+        <v>1.7079300885287607</v>
+      </c>
+      <c r="L91" s="13"/>
+      <c r="M91" s="13"/>
+      <c r="N91" s="6"/>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A92" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B92" s="1">
+        <v>0</v>
+      </c>
+      <c r="C92" s="15">
+        <v>1</v>
+      </c>
+      <c r="D92" s="15"/>
+      <c r="E92" s="15"/>
+      <c r="F92" s="6"/>
+      <c r="G92" s="15">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="H92" s="15"/>
+      <c r="I92" s="15"/>
+      <c r="J92" s="6"/>
+      <c r="K92" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L92" s="13"/>
+      <c r="M92" s="13"/>
+      <c r="N92" s="6"/>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A93" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B93" s="1">
+        <v>0</v>
+      </c>
+      <c r="C93" s="15">
+        <v>1</v>
+      </c>
+      <c r="D93" s="15"/>
+      <c r="E93" s="15"/>
+      <c r="F93" s="6"/>
+      <c r="G93" s="15">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="H93" s="15"/>
+      <c r="I93" s="15"/>
+      <c r="J93" s="6"/>
+      <c r="K93" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L93" s="13"/>
+      <c r="M93" s="13"/>
+      <c r="N93" s="6"/>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A94" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B94" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C94" s="15">
+        <v>-1</v>
+      </c>
+      <c r="D94" s="15"/>
+      <c r="E94" s="15"/>
+      <c r="F94" s="6"/>
+      <c r="G94" s="15">
+        <f t="shared" si="20"/>
+        <v>2</v>
+      </c>
+      <c r="H94" s="15"/>
+      <c r="I94" s="15"/>
+      <c r="J94" s="6"/>
+      <c r="K94" s="13">
+        <f t="shared" ref="K94:K104" si="22">G94/B94</f>
+        <v>-0.66666666666666663</v>
+      </c>
+      <c r="L94" s="13"/>
+      <c r="M94" s="13"/>
+      <c r="N94" s="6"/>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A95" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B95" s="1">
+        <v>1</v>
+      </c>
+      <c r="C95" s="15">
+        <v>7</v>
+      </c>
+      <c r="D95" s="15"/>
+      <c r="E95" s="15"/>
+      <c r="F95" s="6"/>
+      <c r="G95" s="15">
+        <f t="shared" si="20"/>
+        <v>6</v>
+      </c>
+      <c r="H95" s="15"/>
+      <c r="I95" s="15"/>
+      <c r="J95" s="6"/>
+      <c r="K95" s="13">
+        <f t="shared" si="22"/>
+        <v>6</v>
+      </c>
+      <c r="L95" s="13"/>
+      <c r="M95" s="13"/>
+      <c r="N95" s="6"/>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A96" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B96" s="1">
+        <v>7.6160420000000002</v>
+      </c>
+      <c r="C96" s="15">
+        <v>7.1617360000000003</v>
+      </c>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="6"/>
+      <c r="G96" s="15">
+        <f t="shared" si="20"/>
+        <v>-0.45430599999999988</v>
+      </c>
+      <c r="H96" s="15"/>
+      <c r="I96" s="15"/>
+      <c r="J96" s="6"/>
+      <c r="K96" s="13">
+        <f t="shared" si="22"/>
+        <v>-5.9651194150452412E-2</v>
+      </c>
+      <c r="L96" s="13"/>
+      <c r="M96" s="13"/>
+      <c r="N96" s="6"/>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A97" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B97" s="1">
+        <v>8</v>
+      </c>
+      <c r="C97" s="15">
+        <v>7</v>
+      </c>
+      <c r="D97" s="15"/>
+      <c r="E97" s="15"/>
+      <c r="F97" s="6"/>
+      <c r="G97" s="15">
+        <f t="shared" si="20"/>
+        <v>-1</v>
+      </c>
+      <c r="H97" s="15"/>
+      <c r="I97" s="15"/>
+      <c r="J97" s="6"/>
+      <c r="K97" s="13">
+        <f t="shared" si="22"/>
+        <v>-0.125</v>
+      </c>
+      <c r="L97" s="13"/>
+      <c r="M97" s="13"/>
+      <c r="N97" s="6"/>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A98" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B98" s="1">
+        <v>8</v>
+      </c>
+      <c r="C98" s="15">
+        <v>8</v>
+      </c>
+      <c r="D98" s="15"/>
+      <c r="E98" s="15"/>
+      <c r="F98" s="6"/>
+      <c r="G98" s="15">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="H98" s="15"/>
+      <c r="I98" s="15"/>
+      <c r="J98" s="6"/>
+      <c r="K98" s="13">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+      <c r="L98" s="13"/>
+      <c r="M98" s="13"/>
+      <c r="N98" s="6"/>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A99" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B99" s="1">
+        <v>5</v>
+      </c>
+      <c r="C99" s="15">
+        <v>4</v>
+      </c>
+      <c r="D99" s="15"/>
+      <c r="E99" s="15"/>
+      <c r="F99" s="6"/>
+      <c r="G99" s="15">
+        <f t="shared" si="20"/>
+        <v>-1</v>
+      </c>
+      <c r="H99" s="15"/>
+      <c r="I99" s="15"/>
+      <c r="J99" s="6"/>
+      <c r="K99" s="13">
+        <f t="shared" si="22"/>
+        <v>-0.2</v>
+      </c>
+      <c r="L99" s="13"/>
+      <c r="M99" s="13"/>
+      <c r="N99" s="6"/>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A100" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B100" s="1">
+        <v>10234</v>
+      </c>
+      <c r="C100" s="15">
+        <v>6033</v>
+      </c>
+      <c r="D100" s="15"/>
+      <c r="E100" s="15"/>
+      <c r="F100" s="6"/>
+      <c r="G100" s="15">
+        <f t="shared" si="20"/>
+        <v>-4201</v>
+      </c>
+      <c r="H100" s="15"/>
+      <c r="I100" s="15"/>
+      <c r="J100" s="6"/>
+      <c r="K100" s="13">
+        <f t="shared" si="22"/>
+        <v>-0.41049443033027166</v>
+      </c>
+      <c r="L100" s="13"/>
+      <c r="M100" s="13"/>
+      <c r="N100" s="6"/>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A101" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B101" s="5">
+        <v>0.71069444000000004</v>
+      </c>
+      <c r="C101" s="16">
+        <v>0.41895832999999999</v>
+      </c>
+      <c r="D101" s="16"/>
+      <c r="E101" s="16"/>
+      <c r="F101" s="6"/>
+      <c r="G101" s="15">
+        <f t="shared" si="20"/>
+        <v>-0.29173611000000005</v>
+      </c>
+      <c r="H101" s="15"/>
+      <c r="I101" s="15"/>
+      <c r="J101" s="6"/>
+      <c r="K101" s="13">
+        <f t="shared" si="22"/>
+        <v>-0.41049443133394997</v>
+      </c>
+      <c r="L101" s="13"/>
+      <c r="M101" s="13"/>
+      <c r="N101" s="6"/>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A102" s="7"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="12"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="6"/>
+      <c r="G102" s="8"/>
+      <c r="H102" s="8"/>
+      <c r="I102" s="8"/>
+      <c r="J102" s="6"/>
+      <c r="K102" s="8"/>
+      <c r="L102" s="8"/>
+      <c r="M102" s="8"/>
+      <c r="N102" s="6"/>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A103" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B103" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C103" s="19"/>
+      <c r="D103" s="19"/>
+      <c r="E103" s="19"/>
+      <c r="F103" s="6"/>
+      <c r="G103" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H103" s="19"/>
+      <c r="I103" s="19"/>
+      <c r="J103" s="6"/>
+      <c r="K103" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L103" s="19"/>
+      <c r="M103" s="19"/>
+      <c r="N103" s="6"/>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A104" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B104" s="1">
+        <v>4.131875</v>
+      </c>
+      <c r="C104" s="15">
+        <v>3.605556</v>
+      </c>
+      <c r="D104" s="15"/>
+      <c r="E104" s="15"/>
+      <c r="F104" s="6"/>
+      <c r="G104" s="15">
+        <f t="shared" ref="G104:G115" si="23">C104-B104</f>
+        <v>-0.52631899999999998</v>
+      </c>
+      <c r="H104" s="15"/>
+      <c r="I104" s="15"/>
+      <c r="J104" s="6"/>
+      <c r="K104" s="13">
+        <f>G104/B104</f>
+        <v>-0.12738018454091665</v>
+      </c>
+      <c r="L104" s="13"/>
+      <c r="M104" s="13"/>
+      <c r="N104" s="6"/>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A105" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B105" s="1">
+        <v>1.9239580000000001</v>
+      </c>
+      <c r="C105" s="15">
+        <v>1.838889</v>
+      </c>
+      <c r="D105" s="15"/>
+      <c r="E105" s="15"/>
+      <c r="F105" s="6"/>
+      <c r="G105" s="15">
+        <f t="shared" si="23"/>
+        <v>-8.5069000000000061E-2</v>
+      </c>
+      <c r="H105" s="15"/>
+      <c r="I105" s="15"/>
+      <c r="J105" s="6"/>
+      <c r="K105" s="13">
+        <f t="shared" ref="K105:K115" si="24">G105/B105</f>
+        <v>-4.4215622170546372E-2</v>
+      </c>
+      <c r="L105" s="13"/>
+      <c r="M105" s="13"/>
+      <c r="N105" s="6"/>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A106" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B106" s="1">
+        <v>2</v>
+      </c>
+      <c r="C106" s="15">
+        <v>2</v>
+      </c>
+      <c r="D106" s="15"/>
+      <c r="E106" s="15"/>
+      <c r="F106" s="6"/>
+      <c r="G106" s="15">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="H106" s="15"/>
+      <c r="I106" s="15"/>
+      <c r="J106" s="6"/>
+      <c r="K106" s="13">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="L106" s="13"/>
+      <c r="M106" s="13"/>
+      <c r="N106" s="6"/>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A107" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B107" s="1">
+        <v>-2</v>
+      </c>
+      <c r="C107" s="15">
+        <v>-2</v>
+      </c>
+      <c r="D107" s="15"/>
+      <c r="E107" s="15"/>
+      <c r="F107" s="6"/>
+      <c r="G107" s="15">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="H107" s="15"/>
+      <c r="I107" s="15"/>
+      <c r="J107" s="6"/>
+      <c r="K107" s="13">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="L107" s="13"/>
+      <c r="M107" s="13"/>
+      <c r="N107" s="6"/>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A108" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B108" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C108" s="15">
+        <v>-3</v>
+      </c>
+      <c r="D108" s="15"/>
+      <c r="E108" s="15"/>
+      <c r="F108" s="6"/>
+      <c r="G108" s="15">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="H108" s="15"/>
+      <c r="I108" s="15"/>
+      <c r="J108" s="6"/>
+      <c r="K108" s="13">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="L108" s="13"/>
+      <c r="M108" s="13"/>
+      <c r="N108" s="6"/>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A109" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B109" s="1">
+        <v>19</v>
+      </c>
+      <c r="C109" s="15">
+        <v>3</v>
+      </c>
+      <c r="D109" s="15"/>
+      <c r="E109" s="15"/>
+      <c r="F109" s="6"/>
+      <c r="G109" s="15">
+        <f t="shared" si="23"/>
+        <v>-16</v>
+      </c>
+      <c r="H109" s="15"/>
+      <c r="I109" s="15"/>
+      <c r="J109" s="6"/>
+      <c r="K109" s="13">
+        <f t="shared" si="24"/>
+        <v>-0.84210526315789469</v>
+      </c>
+      <c r="L109" s="13"/>
+      <c r="M109" s="13"/>
+      <c r="N109" s="6"/>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A110" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B110" s="1">
+        <v>6.8117359999999998</v>
+      </c>
+      <c r="C110" s="15">
+        <v>6.8386810000000002</v>
+      </c>
+      <c r="D110" s="15"/>
+      <c r="E110" s="15"/>
+      <c r="F110" s="6"/>
+      <c r="G110" s="15">
+        <f t="shared" si="23"/>
+        <v>2.6945000000000441E-2</v>
+      </c>
+      <c r="H110" s="15"/>
+      <c r="I110" s="15"/>
+      <c r="J110" s="6"/>
+      <c r="K110" s="13">
+        <f t="shared" si="24"/>
+        <v>3.9556729738205419E-3</v>
+      </c>
+      <c r="L110" s="13"/>
+      <c r="M110" s="13"/>
+      <c r="N110" s="6"/>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A111" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B111" s="1">
+        <v>7</v>
+      </c>
+      <c r="C111" s="15">
+        <v>7</v>
+      </c>
+      <c r="D111" s="15"/>
+      <c r="E111" s="15"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="15">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="H111" s="15"/>
+      <c r="I111" s="15"/>
+      <c r="J111" s="6"/>
+      <c r="K111" s="13">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="L111" s="13"/>
+      <c r="M111" s="13"/>
+      <c r="N111" s="6"/>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A112" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B112" s="1">
+        <v>8</v>
+      </c>
+      <c r="C112" s="15">
+        <v>8</v>
+      </c>
+      <c r="D112" s="15"/>
+      <c r="E112" s="15"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="15">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="H112" s="15"/>
+      <c r="I112" s="15"/>
+      <c r="J112" s="6"/>
+      <c r="K112" s="13">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="L112" s="13"/>
+      <c r="M112" s="13"/>
+      <c r="N112" s="6"/>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A113" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B113" s="1">
+        <v>4</v>
+      </c>
+      <c r="C113" s="15">
+        <v>5</v>
+      </c>
+      <c r="D113" s="15"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="6"/>
+      <c r="G113" s="15">
+        <f t="shared" si="23"/>
+        <v>1</v>
+      </c>
+      <c r="H113" s="15"/>
+      <c r="I113" s="15"/>
+      <c r="J113" s="6"/>
+      <c r="K113" s="13">
+        <f t="shared" si="24"/>
+        <v>0.25</v>
+      </c>
+      <c r="L113" s="13"/>
+      <c r="M113" s="13"/>
+      <c r="N113" s="6"/>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A114" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B114" s="1">
+        <v>195</v>
+      </c>
+      <c r="C114" s="15">
+        <v>274</v>
+      </c>
+      <c r="D114" s="15"/>
+      <c r="E114" s="15"/>
+      <c r="F114" s="6"/>
+      <c r="G114" s="15">
+        <f t="shared" si="23"/>
+        <v>79</v>
+      </c>
+      <c r="H114" s="15"/>
+      <c r="I114" s="15"/>
+      <c r="J114" s="6"/>
+      <c r="K114" s="13">
+        <f t="shared" si="24"/>
+        <v>0.40512820512820513</v>
+      </c>
+      <c r="L114" s="13"/>
+      <c r="M114" s="13"/>
+      <c r="N114" s="6"/>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A115" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B115" s="5">
+        <v>1.354167E-2</v>
+      </c>
+      <c r="C115" s="13">
+        <v>1.9027780000000001E-2</v>
+      </c>
+      <c r="D115" s="13"/>
+      <c r="E115" s="13"/>
+      <c r="F115" s="6"/>
+      <c r="G115" s="15">
+        <f t="shared" si="23"/>
+        <v>5.4861100000000006E-3</v>
+      </c>
+      <c r="H115" s="15"/>
+      <c r="I115" s="15"/>
+      <c r="J115" s="6"/>
+      <c r="K115" s="13">
+        <f t="shared" si="24"/>
+        <v>0.405128023353102</v>
+      </c>
+      <c r="L115" s="13"/>
+      <c r="M115" s="13"/>
+      <c r="N115" s="6"/>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A116" s="7"/>
+      <c r="B116" s="8"/>
+      <c r="C116" s="8"/>
+      <c r="D116" s="12"/>
+      <c r="E116" s="8"/>
+      <c r="F116" s="6"/>
+      <c r="G116" s="8"/>
+      <c r="H116" s="8"/>
+      <c r="I116" s="8"/>
+      <c r="J116" s="6"/>
+      <c r="K116" s="8"/>
+      <c r="L116" s="8"/>
+      <c r="M116" s="8"/>
+      <c r="N116" s="6"/>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A117" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B117" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C117" s="19"/>
+      <c r="D117" s="19"/>
+      <c r="E117" s="19"/>
+      <c r="F117" s="6"/>
+      <c r="G117" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H117" s="19"/>
+      <c r="I117" s="19"/>
+      <c r="J117" s="6"/>
+      <c r="K117" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L117" s="19"/>
+      <c r="M117" s="19"/>
+      <c r="N117" s="6"/>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A118" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B118" s="1">
+        <v>0.47430600000000001</v>
+      </c>
+      <c r="C118" s="15">
+        <v>2.0395829999999999</v>
+      </c>
+      <c r="D118" s="15"/>
+      <c r="E118" s="15"/>
+      <c r="F118" s="6"/>
+      <c r="G118" s="15">
+        <f t="shared" ref="G118:G129" si="25">C118-B118</f>
+        <v>1.565277</v>
+      </c>
+      <c r="H118" s="15"/>
+      <c r="I118" s="15"/>
+      <c r="J118" s="6"/>
+      <c r="K118" s="13">
+        <f>G118/B118</f>
+        <v>3.3001416806871515</v>
+      </c>
+      <c r="L118" s="13"/>
+      <c r="M118" s="13"/>
+      <c r="N118" s="6"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A119" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B119" s="1">
+        <v>0.346667</v>
+      </c>
+      <c r="C119" s="15">
+        <v>0.93874999999999997</v>
+      </c>
+      <c r="D119" s="15"/>
+      <c r="E119" s="15"/>
+      <c r="F119" s="6"/>
+      <c r="G119" s="15">
+        <f t="shared" si="25"/>
+        <v>0.59208299999999991</v>
+      </c>
+      <c r="H119" s="15"/>
+      <c r="I119" s="15"/>
+      <c r="J119" s="6"/>
+      <c r="K119" s="13">
+        <f t="shared" ref="K119:K129" si="26">G119/B119</f>
+        <v>1.7079300885287607</v>
+      </c>
+      <c r="L119" s="13"/>
+      <c r="M119" s="13"/>
+      <c r="N119" s="6"/>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A120" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B120" s="1">
+        <v>0</v>
+      </c>
+      <c r="C120" s="15">
+        <v>1</v>
+      </c>
+      <c r="D120" s="15"/>
+      <c r="E120" s="15"/>
+      <c r="F120" s="6"/>
+      <c r="G120" s="15">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
+      <c r="H120" s="15"/>
+      <c r="I120" s="15"/>
+      <c r="J120" s="6"/>
+      <c r="K120" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L120" s="13"/>
+      <c r="M120" s="13"/>
+      <c r="N120" s="6"/>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A121" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B121" s="1">
+        <v>0</v>
+      </c>
+      <c r="C121" s="15">
+        <v>1</v>
+      </c>
+      <c r="D121" s="15"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="6"/>
+      <c r="G121" s="15">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
+      <c r="H121" s="15"/>
+      <c r="I121" s="15"/>
+      <c r="J121" s="6"/>
+      <c r="K121" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L121" s="13"/>
+      <c r="M121" s="13"/>
+      <c r="N121" s="6"/>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A122" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B122" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C122" s="15">
+        <v>-1</v>
+      </c>
+      <c r="D122" s="15"/>
+      <c r="E122" s="15"/>
+      <c r="F122" s="6"/>
+      <c r="G122" s="15">
+        <f t="shared" si="25"/>
+        <v>2</v>
+      </c>
+      <c r="H122" s="15"/>
+      <c r="I122" s="15"/>
+      <c r="J122" s="6"/>
+      <c r="K122" s="13">
+        <f t="shared" ref="K122:K132" si="27">G122/B122</f>
+        <v>-0.66666666666666663</v>
+      </c>
+      <c r="L122" s="13"/>
+      <c r="M122" s="13"/>
+      <c r="N122" s="6"/>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A123" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B123" s="1">
+        <v>1</v>
+      </c>
+      <c r="C123" s="15">
+        <v>7</v>
+      </c>
+      <c r="D123" s="15"/>
+      <c r="E123" s="15"/>
+      <c r="F123" s="6"/>
+      <c r="G123" s="15">
+        <f t="shared" si="25"/>
+        <v>6</v>
+      </c>
+      <c r="H123" s="15"/>
+      <c r="I123" s="15"/>
+      <c r="J123" s="6"/>
+      <c r="K123" s="13">
+        <f t="shared" si="27"/>
+        <v>6</v>
+      </c>
+      <c r="L123" s="13"/>
+      <c r="M123" s="13"/>
+      <c r="N123" s="6"/>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A124" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B124" s="1">
+        <v>7.6160420000000002</v>
+      </c>
+      <c r="C124" s="15">
+        <v>7.1617360000000003</v>
+      </c>
+      <c r="D124" s="15"/>
+      <c r="E124" s="15"/>
+      <c r="F124" s="6"/>
+      <c r="G124" s="15">
+        <f t="shared" si="25"/>
+        <v>-0.45430599999999988</v>
+      </c>
+      <c r="H124" s="15"/>
+      <c r="I124" s="15"/>
+      <c r="J124" s="6"/>
+      <c r="K124" s="13">
+        <f t="shared" si="27"/>
+        <v>-5.9651194150452412E-2</v>
+      </c>
+      <c r="L124" s="13"/>
+      <c r="M124" s="13"/>
+      <c r="N124" s="6"/>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A125" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B125" s="1">
+        <v>8</v>
+      </c>
+      <c r="C125" s="15">
+        <v>7</v>
+      </c>
+      <c r="D125" s="15"/>
+      <c r="E125" s="15"/>
+      <c r="F125" s="6"/>
+      <c r="G125" s="15">
+        <f t="shared" si="25"/>
+        <v>-1</v>
+      </c>
+      <c r="H125" s="15"/>
+      <c r="I125" s="15"/>
+      <c r="J125" s="6"/>
+      <c r="K125" s="13">
+        <f t="shared" si="27"/>
+        <v>-0.125</v>
+      </c>
+      <c r="L125" s="13"/>
+      <c r="M125" s="13"/>
+      <c r="N125" s="6"/>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A126" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B126" s="1">
+        <v>8</v>
+      </c>
+      <c r="C126" s="15">
+        <v>8</v>
+      </c>
+      <c r="D126" s="15"/>
+      <c r="E126" s="15"/>
+      <c r="F126" s="6"/>
+      <c r="G126" s="15">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
+      <c r="H126" s="15"/>
+      <c r="I126" s="15"/>
+      <c r="J126" s="6"/>
+      <c r="K126" s="13">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+      <c r="L126" s="13"/>
+      <c r="M126" s="13"/>
+      <c r="N126" s="6"/>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A127" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B127" s="1">
+        <v>5</v>
+      </c>
+      <c r="C127" s="15">
+        <v>4</v>
+      </c>
+      <c r="D127" s="15"/>
+      <c r="E127" s="15"/>
+      <c r="F127" s="6"/>
+      <c r="G127" s="15">
+        <f t="shared" si="25"/>
+        <v>-1</v>
+      </c>
+      <c r="H127" s="15"/>
+      <c r="I127" s="15"/>
+      <c r="J127" s="6"/>
+      <c r="K127" s="13">
+        <f t="shared" si="27"/>
+        <v>-0.2</v>
+      </c>
+      <c r="L127" s="13"/>
+      <c r="M127" s="13"/>
+      <c r="N127" s="6"/>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A128" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B128" s="1">
+        <v>10234</v>
+      </c>
+      <c r="C128" s="15">
+        <v>6033</v>
+      </c>
+      <c r="D128" s="15"/>
+      <c r="E128" s="15"/>
+      <c r="F128" s="6"/>
+      <c r="G128" s="15">
+        <f t="shared" si="25"/>
+        <v>-4201</v>
+      </c>
+      <c r="H128" s="15"/>
+      <c r="I128" s="15"/>
+      <c r="J128" s="6"/>
+      <c r="K128" s="13">
+        <f t="shared" si="27"/>
+        <v>-0.41049443033027166</v>
+      </c>
+      <c r="L128" s="13"/>
+      <c r="M128" s="13"/>
+      <c r="N128" s="6"/>
+    </row>
+    <row r="129" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A129" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B129" s="5">
+        <v>0.71069444000000004</v>
+      </c>
+      <c r="C129" s="16">
+        <v>0.41895832999999999</v>
+      </c>
+      <c r="D129" s="16"/>
+      <c r="E129" s="16"/>
+      <c r="F129" s="6"/>
+      <c r="G129" s="15">
+        <f t="shared" si="25"/>
+        <v>-0.29173611000000005</v>
+      </c>
+      <c r="H129" s="15"/>
+      <c r="I129" s="15"/>
+      <c r="J129" s="6"/>
+      <c r="K129" s="13">
+        <f t="shared" si="27"/>
+        <v>-0.41049443133394997</v>
+      </c>
+      <c r="L129" s="13"/>
+      <c r="M129" s="13"/>
+      <c r="N129" s="6"/>
+    </row>
+    <row r="130" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A130" s="7"/>
+      <c r="B130" s="8"/>
+      <c r="C130" s="8"/>
+      <c r="D130" s="12"/>
+      <c r="E130" s="8"/>
+      <c r="F130" s="6"/>
+      <c r="G130" s="8"/>
+      <c r="H130" s="8"/>
+      <c r="I130" s="8"/>
+      <c r="J130" s="6"/>
+      <c r="K130" s="8"/>
+      <c r="L130" s="8"/>
+      <c r="M130" s="8"/>
+      <c r="N130" s="6"/>
+    </row>
+    <row r="131" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A131" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B131" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C131" s="19"/>
+      <c r="D131" s="19"/>
+      <c r="E131" s="19"/>
+      <c r="F131" s="6"/>
+      <c r="G131" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H131" s="19"/>
+      <c r="I131" s="19"/>
+      <c r="J131" s="6"/>
+      <c r="K131" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="L131" s="19"/>
+      <c r="M131" s="19"/>
+      <c r="N131" s="6"/>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A132" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B132" s="1">
+        <v>4.131875</v>
+      </c>
+      <c r="C132" s="15">
+        <v>3.605556</v>
+      </c>
+      <c r="D132" s="15"/>
+      <c r="E132" s="15"/>
+      <c r="F132" s="6"/>
+      <c r="G132" s="15">
+        <f t="shared" ref="G132:G143" si="28">C132-B132</f>
+        <v>-0.52631899999999998</v>
+      </c>
+      <c r="H132" s="15"/>
+      <c r="I132" s="15"/>
+      <c r="J132" s="6"/>
+      <c r="K132" s="13">
+        <f>G132/B132</f>
+        <v>-0.12738018454091665</v>
+      </c>
+      <c r="L132" s="13"/>
+      <c r="M132" s="13"/>
+      <c r="N132" s="6"/>
+    </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A133" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B133" s="1">
+        <v>1.9239580000000001</v>
+      </c>
+      <c r="C133" s="15">
+        <v>1.838889</v>
+      </c>
+      <c r="D133" s="15"/>
+      <c r="E133" s="15"/>
+      <c r="F133" s="6"/>
+      <c r="G133" s="15">
+        <f t="shared" si="28"/>
+        <v>-8.5069000000000061E-2</v>
+      </c>
+      <c r="H133" s="15"/>
+      <c r="I133" s="15"/>
+      <c r="J133" s="6"/>
+      <c r="K133" s="13">
+        <f t="shared" ref="K133:K143" si="29">G133/B133</f>
+        <v>-4.4215622170546372E-2</v>
+      </c>
+      <c r="L133" s="13"/>
+      <c r="M133" s="13"/>
+      <c r="N133" s="6"/>
+    </row>
+    <row r="134" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A134" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B134" s="1">
+        <v>2</v>
+      </c>
+      <c r="C134" s="15">
+        <v>2</v>
+      </c>
+      <c r="D134" s="15"/>
+      <c r="E134" s="15"/>
+      <c r="F134" s="6"/>
+      <c r="G134" s="15">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="H134" s="15"/>
+      <c r="I134" s="15"/>
+      <c r="J134" s="6"/>
+      <c r="K134" s="13">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="L134" s="13"/>
+      <c r="M134" s="13"/>
+      <c r="N134" s="6"/>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A135" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B135" s="1">
+        <v>-2</v>
+      </c>
+      <c r="C135" s="15">
+        <v>-2</v>
+      </c>
+      <c r="D135" s="15"/>
+      <c r="E135" s="15"/>
+      <c r="F135" s="6"/>
+      <c r="G135" s="15">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="H135" s="15"/>
+      <c r="I135" s="15"/>
+      <c r="J135" s="6"/>
+      <c r="K135" s="13">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="L135" s="13"/>
+      <c r="M135" s="13"/>
+      <c r="N135" s="6"/>
+    </row>
+    <row r="136" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A136" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B136" s="1">
+        <v>-3</v>
+      </c>
+      <c r="C136" s="15">
+        <v>-3</v>
+      </c>
+      <c r="D136" s="15"/>
+      <c r="E136" s="15"/>
+      <c r="F136" s="6"/>
+      <c r="G136" s="15">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="H136" s="15"/>
+      <c r="I136" s="15"/>
+      <c r="J136" s="6"/>
+      <c r="K136" s="13">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="L136" s="13"/>
+      <c r="M136" s="13"/>
+      <c r="N136" s="6"/>
+    </row>
+    <row r="137" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A137" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B137" s="1">
+        <v>19</v>
+      </c>
+      <c r="C137" s="15">
+        <v>3</v>
+      </c>
+      <c r="D137" s="15"/>
+      <c r="E137" s="15"/>
+      <c r="F137" s="6"/>
+      <c r="G137" s="15">
+        <f t="shared" si="28"/>
+        <v>-16</v>
+      </c>
+      <c r="H137" s="15"/>
+      <c r="I137" s="15"/>
+      <c r="J137" s="6"/>
+      <c r="K137" s="13">
+        <f t="shared" si="29"/>
+        <v>-0.84210526315789469</v>
+      </c>
+      <c r="L137" s="13"/>
+      <c r="M137" s="13"/>
+      <c r="N137" s="6"/>
+    </row>
+    <row r="138" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A138" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B138" s="1">
+        <v>6.8117359999999998</v>
+      </c>
+      <c r="C138" s="15">
+        <v>6.8386810000000002</v>
+      </c>
+      <c r="D138" s="15"/>
+      <c r="E138" s="15"/>
+      <c r="F138" s="6"/>
+      <c r="G138" s="15">
+        <f t="shared" si="28"/>
+        <v>2.6945000000000441E-2</v>
+      </c>
+      <c r="H138" s="15"/>
+      <c r="I138" s="15"/>
+      <c r="J138" s="6"/>
+      <c r="K138" s="13">
+        <f t="shared" si="29"/>
+        <v>3.9556729738205419E-3</v>
+      </c>
+      <c r="L138" s="13"/>
+      <c r="M138" s="13"/>
+      <c r="N138" s="6"/>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A139" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B139" s="1">
+        <v>7</v>
+      </c>
+      <c r="C139" s="15">
+        <v>7</v>
+      </c>
+      <c r="D139" s="15"/>
+      <c r="E139" s="15"/>
+      <c r="F139" s="6"/>
+      <c r="G139" s="15">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="H139" s="15"/>
+      <c r="I139" s="15"/>
+      <c r="J139" s="6"/>
+      <c r="K139" s="13">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="L139" s="13"/>
+      <c r="M139" s="13"/>
+      <c r="N139" s="6"/>
+    </row>
+    <row r="140" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B140" s="1">
+        <v>8</v>
+      </c>
+      <c r="C140" s="15">
+        <v>8</v>
+      </c>
+      <c r="D140" s="15"/>
+      <c r="E140" s="15"/>
+      <c r="F140" s="6"/>
+      <c r="G140" s="15">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="H140" s="15"/>
+      <c r="I140" s="15"/>
+      <c r="J140" s="6"/>
+      <c r="K140" s="13">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="L140" s="13"/>
+      <c r="M140" s="13"/>
+      <c r="N140" s="6"/>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A141" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B141" s="1">
+        <v>4</v>
+      </c>
+      <c r="C141" s="15">
+        <v>5</v>
+      </c>
+      <c r="D141" s="15"/>
+      <c r="E141" s="15"/>
+      <c r="F141" s="6"/>
+      <c r="G141" s="15">
+        <f t="shared" si="28"/>
+        <v>1</v>
+      </c>
+      <c r="H141" s="15"/>
+      <c r="I141" s="15"/>
+      <c r="J141" s="6"/>
+      <c r="K141" s="13">
+        <f t="shared" si="29"/>
+        <v>0.25</v>
+      </c>
+      <c r="L141" s="13"/>
+      <c r="M141" s="13"/>
+      <c r="N141" s="6"/>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A142" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B142" s="1">
+        <v>195</v>
+      </c>
+      <c r="C142" s="15">
+        <v>274</v>
+      </c>
+      <c r="D142" s="15"/>
+      <c r="E142" s="15"/>
+      <c r="F142" s="6"/>
+      <c r="G142" s="15">
+        <f t="shared" si="28"/>
+        <v>79</v>
+      </c>
+      <c r="H142" s="15"/>
+      <c r="I142" s="15"/>
+      <c r="J142" s="6"/>
+      <c r="K142" s="13">
+        <f t="shared" si="29"/>
+        <v>0.40512820512820513</v>
+      </c>
+      <c r="L142" s="13"/>
+      <c r="M142" s="13"/>
+      <c r="N142" s="6"/>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A143" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B143" s="5">
+        <v>1.354167E-2</v>
+      </c>
+      <c r="C143" s="13">
+        <v>1.9027780000000001E-2</v>
+      </c>
+      <c r="D143" s="13"/>
+      <c r="E143" s="13"/>
+      <c r="F143" s="6"/>
+      <c r="G143" s="15">
+        <f t="shared" si="28"/>
+        <v>5.4861100000000006E-3</v>
+      </c>
+      <c r="H143" s="15"/>
+      <c r="I143" s="15"/>
+      <c r="J143" s="6"/>
+      <c r="K143" s="13">
+        <f t="shared" si="29"/>
+        <v>0.405128023353102</v>
+      </c>
+      <c r="L143" s="13"/>
+      <c r="M143" s="13"/>
+      <c r="N143" s="6"/>
+    </row>
+    <row r="144" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A144" s="7"/>
+      <c r="B144" s="8"/>
+      <c r="C144" s="8"/>
+      <c r="D144" s="12"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="6"/>
+      <c r="G144" s="8"/>
+      <c r="H144" s="8"/>
+      <c r="I144" s="8"/>
+      <c r="J144" s="6"/>
+      <c r="K144" s="8"/>
+      <c r="L144" s="8"/>
+      <c r="M144" s="8"/>
+      <c r="N144" s="6"/>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A145" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B145" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C145" s="15"/>
+      <c r="D145" s="15"/>
+      <c r="E145" s="15"/>
+      <c r="F145" s="6"/>
+      <c r="G145" s="15">
+        <v>0</v>
+      </c>
+      <c r="H145" s="15"/>
+      <c r="I145" s="15"/>
+      <c r="J145" s="6"/>
+      <c r="K145" s="17">
+        <v>0</v>
+      </c>
+      <c r="L145" s="17"/>
+      <c r="M145" s="17"/>
+      <c r="N145" s="6"/>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A146" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B146" s="15">
+        <v>1</v>
+      </c>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="15"/>
+      <c r="F146" s="6"/>
+      <c r="G146" s="15">
+        <v>0</v>
+      </c>
+      <c r="H146" s="15"/>
+      <c r="I146" s="15"/>
+      <c r="J146" s="6"/>
+      <c r="K146" s="13">
+        <f>G146/B146</f>
+        <v>0</v>
+      </c>
+      <c r="L146" s="13"/>
+      <c r="M146" s="13"/>
+      <c r="N146" s="6"/>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A147" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B147" s="15">
+        <v>278529</v>
+      </c>
+      <c r="C147" s="15"/>
+      <c r="D147" s="15"/>
+      <c r="E147" s="15"/>
+      <c r="F147" s="6"/>
+      <c r="G147" s="15">
+        <v>0</v>
+      </c>
+      <c r="H147" s="15"/>
+      <c r="I147" s="15"/>
+      <c r="J147" s="6"/>
+      <c r="K147" s="13">
+        <f>G147/B147</f>
+        <v>0</v>
+      </c>
+      <c r="L147" s="13"/>
+      <c r="M147" s="13"/>
+      <c r="N147" s="6"/>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A148" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B148" s="15">
+        <v>279694</v>
+      </c>
+      <c r="C148" s="15"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="15"/>
+      <c r="F148" s="6"/>
+      <c r="G148" s="15">
+        <v>0</v>
+      </c>
+      <c r="H148" s="15"/>
+      <c r="I148" s="15"/>
+      <c r="J148" s="6"/>
+      <c r="K148" s="13">
+        <f>G148/B148</f>
+        <v>0</v>
+      </c>
+      <c r="L148" s="13"/>
+      <c r="M148" s="13"/>
+      <c r="N148" s="6"/>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A149" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B149" s="15">
+        <v>295045</v>
+      </c>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15"/>
+      <c r="F149" s="6"/>
+      <c r="G149" s="15">
+        <v>0</v>
+      </c>
+      <c r="H149" s="15"/>
+      <c r="I149" s="15"/>
+      <c r="J149" s="6"/>
+      <c r="K149" s="13">
+        <f>G149/B149</f>
+        <v>0</v>
+      </c>
+      <c r="L149" s="13"/>
+      <c r="M149" s="13"/>
+      <c r="N149" s="6"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A150" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B150" s="15">
+        <f>B149-B146</f>
+        <v>295044</v>
+      </c>
+      <c r="C150" s="15"/>
+      <c r="D150" s="15"/>
+      <c r="E150" s="15"/>
+      <c r="F150" s="6"/>
+      <c r="G150" s="15">
+        <v>0</v>
+      </c>
+      <c r="H150" s="15"/>
+      <c r="I150" s="15"/>
+      <c r="J150" s="6"/>
+      <c r="K150" s="13">
+        <f>G150/B150</f>
+        <v>0</v>
+      </c>
+      <c r="L150" s="13"/>
+      <c r="M150" s="13"/>
+      <c r="N150" s="6"/>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A151" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B151" s="15">
+        <f>B150/(B3*10^3)</f>
+        <v>3.6880500000000001</v>
+      </c>
+      <c r="C151" s="15"/>
+      <c r="D151" s="15"/>
+      <c r="E151" s="1">
+        <f>B150/(E3*10^3)</f>
+        <v>1.47522</v>
+      </c>
+      <c r="F151" s="6"/>
+      <c r="G151" s="15">
+        <v>0</v>
+      </c>
+      <c r="H151" s="15"/>
+      <c r="I151" s="1">
+        <f>E151-B151</f>
+        <v>-2.2128300000000003</v>
+      </c>
+      <c r="J151" s="6"/>
+      <c r="K151" s="13">
+        <v>0</v>
+      </c>
+      <c r="L151" s="13"/>
+      <c r="M151" s="5">
+        <f>I151/B151</f>
+        <v>-0.60000000000000009</v>
+      </c>
+      <c r="N151" s="6"/>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A152" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B152" s="15">
+        <f>B149-B147</f>
+        <v>16516</v>
+      </c>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="15"/>
+      <c r="F152" s="6"/>
+      <c r="G152" s="15">
+        <v>0</v>
+      </c>
+      <c r="H152" s="15"/>
+      <c r="I152" s="15"/>
+      <c r="J152" s="6"/>
+      <c r="K152" s="13">
+        <f>G152/B152</f>
+        <v>0</v>
+      </c>
+      <c r="L152" s="13"/>
+      <c r="M152" s="13"/>
+      <c r="N152" s="6"/>
+    </row>
+    <row r="153" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A153" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B153" s="15">
+        <f>B152/B3</f>
+        <v>206.45</v>
+      </c>
+      <c r="C153" s="15"/>
+      <c r="D153" s="15"/>
+      <c r="E153" s="1">
+        <f>B152/E3</f>
+        <v>82.58</v>
+      </c>
+      <c r="F153" s="6"/>
+      <c r="G153" s="15">
+        <v>0</v>
+      </c>
+      <c r="H153" s="15"/>
+      <c r="I153" s="1">
+        <f>E153-B153</f>
+        <v>-123.86999999999999</v>
+      </c>
+      <c r="J153" s="6"/>
+      <c r="K153" s="13">
+        <v>0</v>
+      </c>
+      <c r="L153" s="13"/>
+      <c r="M153" s="5">
+        <f>I153/B153</f>
+        <v>-0.6</v>
+      </c>
+      <c r="N153" s="6"/>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A154" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B154" s="1">
+        <f>B12*B151</f>
+        <v>2938.4169569999999</v>
+      </c>
+      <c r="C154" s="1">
+        <f>C12*B151</f>
+        <v>2899.5817905000004</v>
+      </c>
+      <c r="D154" s="11">
+        <f>D12*B151</f>
+        <v>2987.4311414999997</v>
+      </c>
+      <c r="E154" s="1">
+        <f t="shared" ref="E154" si="30">E12*E151</f>
+        <v>2045.7023262</v>
+      </c>
+      <c r="F154" s="6"/>
+      <c r="G154" s="1">
+        <f>C154-B154</f>
+        <v>-38.835166499999559</v>
+      </c>
+      <c r="H154" s="1">
+        <f>D154-B154</f>
+        <v>49.014184499999828</v>
+      </c>
+      <c r="I154" s="1">
+        <f>E154-B154</f>
+        <v>-892.7146307999999</v>
+      </c>
+      <c r="J154" s="6"/>
+      <c r="K154" s="5">
+        <f>G154/B154</f>
+        <v>-1.3216356653362302E-2</v>
+      </c>
+      <c r="L154" s="5">
+        <f>H154/B154</f>
+        <v>1.6680472927178194E-2</v>
+      </c>
+      <c r="M154" s="5"/>
+      <c r="N154" s="6"/>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A155" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B155" s="15">
+        <f>1/(B151/1000)</f>
+        <v>271.1459985629262</v>
+      </c>
+      <c r="C155" s="15"/>
+      <c r="D155" s="15"/>
+      <c r="E155" s="1">
+        <f>1/(E151/1000)</f>
+        <v>677.86499640731552</v>
+      </c>
+      <c r="F155" s="6"/>
+      <c r="G155" s="15">
+        <v>0</v>
+      </c>
+      <c r="H155" s="15"/>
+      <c r="I155" s="1">
+        <f>E155-B155</f>
+        <v>406.71899784438932</v>
+      </c>
+      <c r="J155" s="6"/>
+      <c r="K155" s="13">
+        <v>0</v>
+      </c>
+      <c r="L155" s="13"/>
+      <c r="M155" s="5">
+        <f>I155/B155</f>
         <v>1.5</v>
       </c>
-      <c r="N69" s="6"/>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A70" s="7"/>
-      <c r="B70" s="8"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="12"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="6"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-      <c r="I70" s="8"/>
-      <c r="J70" s="6"/>
-      <c r="K70" s="8"/>
-      <c r="L70" s="8"/>
-      <c r="M70" s="8"/>
-      <c r="N70" s="6"/>
+      <c r="N155" s="6"/>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A156" s="7"/>
+      <c r="B156" s="8"/>
+      <c r="C156" s="8"/>
+      <c r="D156" s="12"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="6"/>
+      <c r="G156" s="8"/>
+      <c r="H156" s="8"/>
+      <c r="I156" s="8"/>
+      <c r="J156" s="6"/>
+      <c r="K156" s="8"/>
+      <c r="L156" s="8"/>
+      <c r="M156" s="8"/>
+      <c r="N156" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="113">
-    <mergeCell ref="K34:M34"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="K1:M1"/>
+  <mergeCells count="353">
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="K86:M86"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="G87:I87"/>
+    <mergeCell ref="K87:M87"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="G83:I83"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="K84:M84"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="K85:M85"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="K80:M80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="K81:M81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="G77:I77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="K67:M67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="K68:M68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="K69:M69"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="K114:M114"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="K115:M115"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:I62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="K63:M63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="G65:I65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="K66:M66"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="K111:M111"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="G113:I113"/>
+    <mergeCell ref="K113:M113"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="G108:I108"/>
+    <mergeCell ref="K108:M108"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="K109:M109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="K110:M110"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="K105:M105"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="K106:M106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="G107:I107"/>
+    <mergeCell ref="K107:M107"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="K98:M98"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="K100:M100"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="K95:M95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="K96:M96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="K97:M97"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="K92:M92"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="K93:M93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="K94:M94"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="G89:I89"/>
+    <mergeCell ref="K89:M89"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="G90:I90"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="C141:E141"/>
+    <mergeCell ref="G141:I141"/>
+    <mergeCell ref="K141:M141"/>
+    <mergeCell ref="C142:E142"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="K142:M142"/>
+    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="K143:M143"/>
+    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="K138:M138"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="K139:M139"/>
+    <mergeCell ref="C140:E140"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="K140:M140"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="K135:M135"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="G136:I136"/>
+    <mergeCell ref="K136:M136"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="G137:I137"/>
+    <mergeCell ref="K137:M137"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="K132:M132"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="K133:M133"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="K134:M134"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="K128:M128"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="K129:M129"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="G131:I131"/>
+    <mergeCell ref="K131:M131"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="G125:I125"/>
+    <mergeCell ref="K125:M125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="K126:M126"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="K127:M127"/>
+    <mergeCell ref="K121:M121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="K123:M123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="G124:I124"/>
+    <mergeCell ref="K124:M124"/>
+    <mergeCell ref="K146:M146"/>
+    <mergeCell ref="K147:M147"/>
+    <mergeCell ref="K148:M148"/>
+    <mergeCell ref="K149:M149"/>
+    <mergeCell ref="K150:M150"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="G33:I33"/>
     <mergeCell ref="K33:M33"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="B47:E47"/>
     <mergeCell ref="G47:I47"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B67:D67"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="K118:M118"/>
+    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="G119:I119"/>
+    <mergeCell ref="K119:M119"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="K120:M120"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="K145:M145"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="G153:H153"/>
+    <mergeCell ref="G151:H151"/>
+    <mergeCell ref="G155:H155"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="K59:M59"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="G147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="K152:M152"/>
+    <mergeCell ref="K151:L151"/>
+    <mergeCell ref="K153:L153"/>
+    <mergeCell ref="K155:L155"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="B153:D153"/>
+    <mergeCell ref="B155:D155"/>
     <mergeCell ref="G34:I34"/>
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="G36:I36"/>
@@ -3096,59 +5649,68 @@
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="G43:I43"/>
     <mergeCell ref="G44:I44"/>
-    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="G45:I45"/>
     <mergeCell ref="C40:E40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="C42:E42"/>
     <mergeCell ref="C43:E43"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="B151:D151"/>
+    <mergeCell ref="G48:I48"/>
     <mergeCell ref="G49:I49"/>
     <mergeCell ref="G50:I50"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="K40:M40"/>
     <mergeCell ref="K41:M41"/>
+    <mergeCell ref="G56:I56"/>
     <mergeCell ref="K42:M42"/>
     <mergeCell ref="K43:M43"/>
     <mergeCell ref="K44:M44"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="G60:I60"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="K66:M66"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="K67:L67"/>
-    <mergeCell ref="K69:L69"/>
-    <mergeCell ref="K60:M60"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="K63:M63"/>
-    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>